<commit_message>
N27 banco de mensajes: orden de hojas por lectura
Instrucciones, Por situacion y el banco de 108 mensajes al final, que es
material de consulta y no por donde se empieza.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/recursos/impulso-n27-banco-mensajes-tipo.xlsx
+++ b/public/recursos/impulso-n27-banco-mensajes-tipo.xlsx
@@ -8,11 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensajes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por situación" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por situación" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensajes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mensajes'!$A$4:$H$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mensajes'!$A$4:$H$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -127,15 +127,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -151,7 +152,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -743,6 +743,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Por situación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuántos mensajes hay de cada tipo y por dónde empezar con el equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Situación</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Mensajes</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Primera fila en 'Mensajes'</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Por dónde empezar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Dudas sobre el genérico</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Fila 5</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Es la consulta que más veces se contesta distinto en la misma farmacia. Acordadla primero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Primera dispensación de un crónico</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Fila 14</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Aquí se juega la adherencia de los próximos meses. Vale la pena la versión larga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>La novedad que ha visto en televisión o redes</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Fila 23</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>El riesgo es quedar por encima del paciente. Acordad el tono antes que el contenido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Cuando la respuesta es que no</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Fila 32</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>El momento que más desiguala a un equipo. Si solo escribís un bloque, que sea este.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Dejar de fumar</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Fila 41</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Consulta larga en un mostrador con cola: acordad cuándo se cita para otro momento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Complementos y probióticos</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Fila 50</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Cuidado con prometer. Revisad juntos la línea entre acompañar y colocar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Dermofarmacia y consulta de piel</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Fila 59</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Definid entre todos dónde está el límite para derivar al médico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>El precio y la comparación con internet</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Fila 68</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Se responde sin defenderse. Practicadlo en voz alta, cambia mucho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>No lo tenemos ahora mismo</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Fila 77</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Lo importante no es la falta, es que el paciente se vaya sabiendo qué pasa y cuándo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Mayores y polimedicación</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Fila 86</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Bajad el ritmo y comprobad que se ha entendido. Es la parte que más se olvida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Cuando hay que derivar al médico</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Fila 95</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Acordad las señales de alarma por escrito. Es lo único que no admite estilo propio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Quejas y momentos incómodos</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Fila 104</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Reconocer el hecho no es dar la razón. Ensayadlo con dos personas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Total: 108 mensajes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -814,10 +1122,10 @@
       </c>
     </row>
     <row r="5" ht="74" customHeight="1">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
@@ -842,62 +1150,62 @@
           <t>Antes de autorizarse, un genérico tiene que demostrar que actúa en el cuerpo igual que el medicamento original. Lo único que cambia es el laboratorio que lo fabrica y, a veces, el aspecto de la caja o el comprimido. El precio es más bajo porque el laboratorio no paga la investigación inicial, que ya está amortizada por el medicamento de referencia. Si alguna vez notas algo distinto con un cambio de marca, coméntalo en la farmacia, aunque no es lo habitual.</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>No respondas con un 'da igual cuál te lleves' sin explicar nada, porque suena a que no te lo has tomado en serio.</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>Si el paciente dice que un genérico concreto le sienta peor, anota el nombre y coméntalo con el farmacéutico antes de darlo por sensación.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="74" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>«¿Por qué hoy me dais uno distinto al de la última vez?»</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Depende de qué genérico tenga en stock el almacén ese día, el principio activo es el mismo.</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>La farmacia dispensa el genérico que tiene disponible en ese momento, y puede cambiar de una compra a otra. El principio activo, la dosis y el efecto son los mismos, cambia solo el fabricante.</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>En cada pedido a nuestro proveedor recibimos el genérico que hay disponible en ese momento, que no siempre es el mismo laboratorio. Eso hace que la caja cambie de forma, de color o de nombre comercial de una vez a otra. Lo que no cambia nunca es el principio activo ni la dosis que te recetó el médico. Si te resulta confuso, podemos anotarte en la ficha qué laboratorio llevas cada vez para que lo identifiques mejor.</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>No le quites importancia con un 'es lo mismo, no te preocupes' seco, porque el paciente busca entender el cambio, no que lo ignoren.</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>Para pacientes mayores o polimedicados conviene anotar el laboratorio en la ficha o en la caja, así evitas confusiones en casa.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="74" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
@@ -922,62 +1230,62 @@
           <t>Por supuesto, puedes pedir siempre la marca, es tu dinero y tu decisión. Lo que quiero que sepas es que el genérico no es una versión inferior: pasa los mismos controles de calidad y demuestra que actúa igual en el cuerpo antes de salir a la venta. La desconfianza viene muchas veces de la idea de que lo barato es peor, pero aquí el precio bajo no significa menos calidad. Dicho esto, si te sientes más tranquilo con la marca, nosotros te la preparamos sin ningún problema.</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>No discutas ni intentes convencer al paciente de que está equivocado, respeta su decisión y explica sin insistir.</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Comprueba antes si su seguro o mutua cubre solo el genérico, porque en algunos casos la marca no está financiada igual.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="74" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>«¿Los genéricos llevan menos cantidad del principio activo?»</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>No, llevan exactamente la misma cantidad y la misma dosis que el original.</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Llevan la misma cantidad de principio activo y la misma dosis, eso es obligatorio para que se apruebe como genérico. Lo que puede cambiar son los excipientes, que no tienen efecto terapéutico.</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>No, la cantidad de principio activo y la dosis tienen que ser exactamente iguales a las del medicamento original, eso lo exige la normativa antes de autorizar el genérico. Lo que sí puede variar son los excipientes, es decir, los componentes que dan forma al comprimido o al jarabe pero que no actúan en la enfermedad. Por eso, en personas alérgicas a algún excipiente concreto, conviene revisar el prospecto al cambiar de laboratorio. Fuera de ese caso puntual, el efecto que notarás es el mismo.</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>No des por hecho que la duda es infundada; explicar la diferencia entre principio activo y excipiente resuelve la preocupación real.</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Si el paciente tiene alergias conocidas a excipientes, comprueba el prospecto del genérico concreto antes de dispensarlo.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="74" customHeight="1">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
@@ -1002,62 +1310,62 @@
           <t>La receta electrónica indica si el médico ha marcado que no se puede sustituir el medicamento; si no lo ha marcado, la farmacia tiene margen para dispensar el genérico equivalente. Es una práctica habitual y regulada, no una decisión nuestra al azar. Si para ti es importante llevarte exactamente la marca que puso el médico, lo comentas y te la buscamos, aunque a veces implique un coste distinto. Y si tienes dudas de fondo sobre el cambio, es buen momento para preguntárselo también a tu médico en la próxima visita.</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>No respondas con un genérico 'es que así es la ley' sin más, porque suena a excusa y no explica la sustitución.</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>Si la receta lleva marcada la casilla de sustitución no permitida, no se puede cambiar el medicamento bajo ningún concepto.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="74" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>«Cambiáis de genérico cada vez que vengo, ¿eso es normal?»</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Sí, depende del laboratorio que tengamos disponible en cada pedido, es normal.</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Es normal, la farmacia recibe el genérico según disponibilidad del proveedor y puede variar de compra en compra. El principio activo y la dosis se mantienen siempre iguales.</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>Es normal y no depende de nosotros: recibimos el genérico que hay disponible en cada pedido, y varios laboratorios fabrican el mismo principio activo. Eso hace que la caja cambie de aspecto de una visita a otra, aunque el medicamento que llevas dentro sea equivalente. Entiendo que pueda resultar confuso, sobre todo si tomas varias pastillas distintas. Si quieres, apuntamos en tu ficha qué presentación llevas cada vez para que la reconozcas mejor en casa.</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>No lo minimices con un 'sí, sí, es igual' automático, porque para pacientes con varias cajas parecidas el cambio genera confusión real.</t>
         </is>
       </c>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="H10" s="15" t="inlineStr">
         <is>
           <t>En pacientes polimedicados o mayores, ofrece siempre apuntar el laboratorio en la caja o en un pastillero para evitar errores de toma.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="74" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
@@ -1082,62 +1390,62 @@
           <t>Nada de eso, la elección entre genérico y marca no tiene relación con lo que se vende más o menos en la farmacia. El genérico es un medicamento que ha pasado por la misma autoridad sanitaria que el original y ha tenido que demostrar que actúa igual en el cuerpo. Se fabrica y se dispensa igual, con los mismos controles de calidad en cada lote. La única diferencia real es el laboratorio que lo produce y, por eso, el precio.</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>No te rías de la pregunta ni la despaches con un 'qué cosas dicen por ahí', porque detrás hay una duda real sobre la calidad.</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>Si el paciente sigue desconfiando, ofrécele el prospecto del genérico para que compare la ficha técnica con la del original.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="74" customHeight="1">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>«Con este genérico me ha sentado peor que con el de siempre»</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Cuéntame qué notaste exactamente, puede depender del excipiente o de otra causa.</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Es raro que cambie el efecto real, porque el principio activo es el mismo, pero cuéntame qué síntoma has notado. A veces influye algún excipiente concreto o simplemente coincide con otra causa.</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>El principio activo es idéntico, así que el efecto terapéutico no debería cambiar de un genérico a otro. Cuéntame exactamente qué has notado: si es algo digestivo, cutáneo o de otro tipo, porque a veces sí influye algún excipiente distinto en personas sensibles. También puede ser una coincidencia con otra causa, como otro medicamento nuevo o algo que hayas comido. Si el síntoma es claro y se repite, lo anotamos y, si hace falta, lo consultamos con tu médico.</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>No descartes la sensación del paciente con un 'eso es imposible', escúchalo primero aunque el principio activo sea el mismo.</t>
         </is>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Si el síntoma es grave o persiste, deriva al médico; si es leve y puntual, anótalo en la ficha por si se repite con el mismo laboratorio.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="74" customHeight="1">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Dudas sobre el genérico</t>
         </is>
@@ -1162,62 +1470,62 @@
           <t>Entiendo la desconfianza, pero el precio bajo tiene una explicación sencilla: desarrollar un medicamento nuevo cuesta muchos años de investigación, y esa inversión la asume el laboratorio que lo crea primero. Cuando esa protección termina, otros laboratorios pueden fabricar el mismo principio activo sin repetir esa investigación, y por eso lo venden más barato. Pasa por los mismos controles de calidad y por la misma autoridad sanitaria antes de llegar a la farmacia. Barato aquí no significa peor, significa que no arrastra ese coste inicial.</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>No te quedes callado ante la sospecha ni respondas solo 'no', explica de dónde viene el precio para que la duda no se quede sin resolver.</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Es una buena ocasión para explicar qué es la patente y por qué caduca, ayuda a que la duda no vuelva en la próxima visita.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="74" customHeight="1">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>«Me acaban de diagnosticar y no sé ni cómo tomar esto»</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Tranquilo, te explico ahora mismo cuándo y cómo tomarlo paso a paso.</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>No pasa nada, es normal sentirse perdido al principio. Vamos a ver juntos la pauta, a qué hora te viene mejor tomarlo y qué hacer si algún día se te olvida.</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Es totalmente normal sentirse perdido el primer día, a casi todo el mundo le pasa. Vamos a repasar juntos la pauta que te ha dejado el médico: cuántas veces al día, si es con comida o en ayunas, y a qué hora te resulta más fácil acordarte. Te doy también un par de trucos, como asociarlo a un hábito diario, por ejemplo el cepillado de dientes. Y quédate tranquilo, si tienes cualquier duda en los próximos días puedes volver o llamarnos, no hace falta esperar a la siguiente visita.</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>No sueltes toda la información técnica de golpe, abruma más de lo que ayuda; ve paso a paso y comprueba que lo va entendiendo.</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="15" t="inlineStr">
         <is>
           <t>Aprovecha esta primera dispensación para preguntar si toma otra medicación o tiene alergias, es el mejor momento para detectar interacciones.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="74" customHeight="1">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
@@ -1242,62 +1550,62 @@
           <t>Eso depende mucho de cada caso: hay tratamientos que se ajustan o se retiran con el tiempo, y otros que se mantienen porque controlan algo de forma continua. Quien mejor puede decírtelo es tu médico, valorando cómo evolucionas en las revisiones. Desde la farmacia lo que podemos hacer es ayudarte a que la toma sea cómoda y no se te olvide, porque eso influye mucho en el resultado. Si con el tiempo te surgen dudas sobre si sigue haciendo falta, es buena pregunta para la próxima cita.</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>No des un 'sí, para siempre' ni un 'no, ya verás' sin base, esa respuesta le corresponde al médico, no la inventes en el mostrador.</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>Nunca sugieras que se puede dejar sin más si mejora; recuérdale siempre que cualquier cambio de pauta lo decide el médico.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="74" customHeight="1">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>«¿Qué pasa si un día se me olvida tomarlo?»</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Depende del medicamento, dime cuál es y te digo exactamente qué hacer.</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Cada medicamento tiene su propia norma para las dosis olvidadas, así que dime cuál tomas y te lo concreto. Como norma general, nunca se toma una dosis doble para compensar sin habértelo dicho antes.</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>La respuesta cambia según el medicamento, así que te la concreto para el tuyo, no vale una norma única para todos. Como idea general, si te acuerdas poco después la tomas y sigues igual; si ya está cerca de la siguiente dosis, en muchos casos se salta esa toma. Lo que casi nunca se hace es tomar doble dosis para compensar el olvido. Te lo anoto para que lo tengas siempre a mano en casa.</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>No des una regla genérica de 'tómalo en cuanto te acuerdes' para cualquier medicamento, algunos tienen normas distintas y puede ser un error.</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H16" s="15" t="inlineStr">
         <is>
           <t>Anota la pauta concreta de olvido en la caja o en el prospecto del paciente, sobre todo si toma varios medicamentos distintos.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="74" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
@@ -1322,62 +1630,62 @@
           <t>Cada medicamento tiene su propia recomendación sobre el momento de la toma, así que te lo confirmo exactamente para el que llevas. Algunos se absorben mejor en ayunas, otros necesitan algo de comida para no irritar el estómago, y unos pocos incluso interaccionan con la cafeína o los lácteos. Si no te especifica nada el prospecto, lo normal es que puedas tomarlo con el desayuno sin problema. Lo importante es mantener siempre el mismo horario cada día, más que el café en sí.</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>No contestes 'con lo que quieras' sin comprobarlo, algunos principios activos sí pierden eficacia o dan molestias si se toman mal.</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>Comprueba siempre el prospecto o la ficha técnica del medicamento concreto antes de confirmar si puede tomarse con cafeína o lácteos.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="74" customHeight="1">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>«Me han recetado dos pastillas nuevas, ¿interfieren entre ellas?»</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Déjame revisarlo con calma, dime los dos nombres y te lo confirmo ahora.</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Es justo lo que tengo que comprobar antes de dártelas, así que dame un momento para revisar los dos medicamentos juntos. Si hay algo que vigilar, te lo explico ahora mismo.</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Muy buena pregunta, y es justo parte de mi trabajo antes de entregarte cualquier medicación nueva. Voy a comprobar los dos principios activos juntos y también los que ya tomes de antes, por si hay alguna combinación que requiera espaciar las tomas o vigilar algún síntoma. La mayoría de las veces se pueden tomar sin problema, pero prefiero confirmarlo con datos y no de memoria. Si detecto algo relevante, te lo explico y, si hace falta, lo comentamos con tu médico.</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>No contestes 'seguro que no pasa nada' sin comprobarlo en la ficha del paciente, es justo el tipo de error que hay que evitar.</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>Consulta siempre la ficha completa de medicación del paciente, no solo lo que se lleva ese día, para detectar interacciones reales.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="74" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
@@ -1402,62 +1710,62 @@
           <t>Como cualquier medicamento, este puede dar algún efecto secundario, aunque la mayoría de las personas lo toleran bien. Los más frecuentes suelen ser leves, como molestias digestivas o algo de somnolencia los primeros días, y normalmente van desapareciendo. Hay otros menos comunes que sí conviene vigilar, y te los señalo para que sepas identificarlos si aparecen. Si notas algo que te preocupa, sobre todo algo repentino o intenso, no esperes a la próxima revisión, coméntalo antes.</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>No leas el prospecto entero al pie de la letra, asusta más de lo que informa; destaca solo lo relevante para ese paciente.</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>Señala claramente cuáles son señales de alarma que requieren ir a urgencias o llamar al médico, no solo molestias leves.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="74" customHeight="1">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>«No quiero depender de una pastilla el resto de mi vida»</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Lo entiendo, coméntaselo a tu médico, hay hábitos que también ayudan al tratamiento.</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Es una reacción muy común, a nadie le gusta empezar un tratamiento largo. Coméntaselo a tu médico, porque en algunos casos ciertos cambios de hábitos ayudan a controlar mejor la enfermedad, aunque eso lo valora él, no yo.</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>Es una reacción muy humana, empezar un tratamiento para toda la vida cuesta de aceptar al principio. Lo que te puedo decir es que en muchos casos el medicamento no sustituye tus hábitos, los acompaña: la alimentación, el ejercicio o el descanso también influyen en cómo evoluciona la enfermedad. Coméntale esa preocupación a tu médico, porque él es quien puede decirte si con el tiempo hay margen para ajustar la pauta. Mientras tanto, tomarlo bien ahora es lo que más ayuda a que las cosas vayan mejor.</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>No le digas que 'no tiene otra opción', suena a sentencia; valida la incomodidad y deriva la decisión de fondo al médico.</t>
         </is>
       </c>
-      <c r="H20" s="14" t="inlineStr">
+      <c r="H20" s="15" t="inlineStr">
         <is>
           <t>Nunca insinúes que puede sustituir el medicamento por hábitos de vida sin que lo indique el médico, aunque estos ayuden.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="74" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
@@ -1482,62 +1790,62 @@
           <t>Es una trampa muy común: te encuentras bien porque el medicamento está controlando la enfermedad por dentro, no porque ya no haga falta. Si lo dejas por tu cuenta, puede que no notes nada al principio y que el problema vuelva semanas después, a veces peor que antes. Esa decisión la tiene que tomar tu médico, valorando pruebas, no cómo te sientas un día concreto. Coméntaselo en la próxima revisión, es una pregunta totalmente legítima.</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>No le des la razón para tranquilizarlo en el momento; dejar un tratamiento crónico sin control médico puede tener consecuencias serias.</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>Si detectas que el paciente ya ha reducido o dejado la medicación por su cuenta, anímalo a decírselo a su médico cuanto antes, sin juzgarlo.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="74" customHeight="1">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Primera dispensación de un crónico</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>«Es la primera vez que tomo algo para esto y me da un poco de miedo»</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Es normal, vamos despacio y te explico todo lo que necesitas saber.</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>Es totalmente normal sentir eso al principio, casi todo el mundo pasa por lo mismo. Vamos a repasar con calma cómo tomarlo, qué esperar los primeros días y a quién llamar si tienes dudas.</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>El miedo al principio es muy normal, sobre todo con una enfermedad nueva. Vamos despacio: te explico cómo y cuándo tomarlo, qué notar los primeros días y qué es esperable frente a lo que no lo es. También te digo cómo contactar con la farmacia si te surge una duda entre visita y visita al médico. Con los días, la rutina de tomarlo se vuelve mucho más sencilla de lo que parece ahora.</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G22" s="15" t="inlineStr">
         <is>
           <t>No le quites importancia con un 'no es nada' rápido, el miedo es real y necesita información concreta, no una frase hecha.</t>
         </is>
       </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="H22" s="15" t="inlineStr">
         <is>
           <t>Aprovecha para preguntar si vive solo o tiene apoyo en casa, influye en cómo planteamos el seguimiento de la primera semana.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="74" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
@@ -1562,62 +1870,62 @@
           <t>Ese tipo de anuncios prometen resultados que ningún producto puede dar por sí solo, y menos mientras duermes. La pérdida de peso depende de muchos factores, sobre todo la alimentación y la actividad física, y ahí no hay atajo en una cápsula. Algunos suplementos pueden acompañar un cambio de hábitos, pero nunca sustituirlo ni garantizar el resultado por su cuenta. Si de verdad quieres bajar de peso de forma segura, te puedo orientar sobre opciones serias o derivarte a quien valore tu caso concreto.</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>No te limites a decir 'eso es mentira' y cortar la conversación, explica por qué no funciona para que no lo compre en otro sitio.</t>
         </is>
       </c>
-      <c r="H23" s="10" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>Si el paciente toma otra medicación, revisa siempre el suplemento antes de dar el visto bueno, algunos interaccionan aunque parezcan inofensivos.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="74" customHeight="1">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>«En Instagram dicen que esta planta baja el colesterol en una semana»</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>En una semana no se baja el colesterol, desconfía de esa promesa de redes.</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Bajar el colesterol lleva más de una semana y depende de varios factores, no solo de una planta. Hay plantas que pueden ayudar como complemento de la dieta, pero nunca de forma tan rápida ni sustituyendo el tratamiento si lo tienes.</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>El colesterol no baja en una semana con nada, ni con plantas ni con dietas milagro, esos plazos son marketing puro. Hay complementos con cierta base, como algunas fibras o fitoesteroles, que pueden ayudar dentro de una alimentación cuidada, pero su efecto es progresivo y modesto, no una solución rápida. Si ya tomas medicación para el colesterol, nunca la sustituyas por un suplemento sin hablarlo antes con tu médico. Si aún no tomas nada, mide primero con una analítica cómo lo tienes, no te fíes solo de un vídeo.</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>No valides la fuente solo porque 'lo he visto en redes', pregunta qué planta es exactamente antes de opinar.</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>Si toma estatinas u otro hipolipemiante, comprueba siempre interacciones antes de aprobar cualquier planta o suplemento adicional.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="74" customHeight="1">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
@@ -1642,62 +1950,62 @@
           <t>Entiendo que si a alguien cercano le ha ido bien apetezca probarlo, pero lo que funciona en una persona no garantiza nada en otra, no es la misma edad ni el mismo historial. Tu médico te ha recetado ese tratamiento valorando tu caso concreto, con datos que tu cuñado no tiene por qué conocer. Cambiarlo por comparación puede hacer que lo tuyo no se controle bien. Si de verdad no notas mejoría, coméntaselo al médico, pero no lo sustituyas por tu cuenta.</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>No te pongas a discutir con el cuñado ausente ni ridiculices el consejo, redirige con respeto hacia el criterio del médico.</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Pregunta con curiosidad qué es exactamente lo que le recomendaron, a veces es un hábito razonable y otras un producto de riesgo real.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="74" customHeight="1">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>«¿Tenéis el producto que sale en el anuncio de la tele?»</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Dime qué necesitas exactamente y te busco algo equivalente que sí tengamos aquí.</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>No sabría decirte sin más detalle, cuéntame qué problema quieres resolver y te oriento sobre qué opciones tenemos aquí, sean o no la marca del anuncio.</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Los anuncios suelen centrarse en un nombre concreto, pero lo importante es para qué lo quieres, no la marca en sí. Cuéntame qué molestia o qué necesidad tienes detrás del anuncio y te oriento sobre qué opciones manejamos aquí, con el mismo tipo de ingrediente o una alternativa razonable. A veces el producto de la tele es correcto para ese uso, y otras veces hay opciones más adecuadas para tu caso concreto que no salen en ningún anuncio. Así eliges con información, no solo porque lo hayas visto repetido.</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G26" s="15" t="inlineStr">
         <is>
           <t>No digas simplemente 'eso no lo tenemos' sin más, cierra la conversación en falso; pregunta primero qué necesita de verdad.</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>Si el producto anunciado exige receta o tiene contraindicaciones, es el momento de decirlo antes de que lo busque en otro sitio sin control.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="74" customHeight="1">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
@@ -1722,62 +2030,62 @@
           <t>La palabra 'rejuvenecer' vende mucho, pero ningún suplemento revierte el paso del tiempo en la piel desde dentro. Tomar colágeno puede acompañar un cuidado general, junto con protección solar y buena alimentación, pero su efecto real es mucho más modesto que el del anuncio. El envejecimiento de la piel depende de la genética, el sol acumulado y el tabaco, factores que ningún suplemento compensa por sí solo. Si buscas cuidar tu piel, te oriento sobre qué tiene sentido añadir a tu rutina.</t>
         </is>
       </c>
-      <c r="G27" s="10" t="inlineStr">
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>No confirmes la palabra 'rejuvenece' asintiendo sin más, refuerza una expectativa que ningún producto puede cumplir.</t>
         </is>
       </c>
-      <c r="H27" s="10" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>Si el paciente tiene alguna alergia o toma anticoagulantes, revisa el suplemento antes de recomendarlo, no todo colágeno es igual de inocuo.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="74" customHeight="1">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>«Una influencer toma esto cada mañana y dice que no se resfría nunca»</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Ningún producto evita todos los resfriados, eso no es verificable ni realista.</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Que a alguien no le dé un resfriado en un tiempo no prueba nada sobre un producto concreto, influyen muchas cosas más. No hay ningún suplemento que garantice inmunidad total frente a los catarros.</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>El testimonio de una persona no prueba nada, puede que simplemente no se haya cruzado con el virus, o que influyan el descanso o el contacto con más o menos gente. Ningún suplemento garantiza que no te vayas a resfriar, eso depende del sistema inmunitario y de la exposición. Algunas vitaminas pueden tener un papel de apoyo si hay una carencia real, pero no un efecto de blindaje total. Si te interesa cuidar las defensas, hay hábitos con más base que un solo producto de mañana.</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>No te burles del influencer ni del paciente por creerle, resta credibilidad con datos, no con desprecio hacia la fuente.</t>
         </is>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H28" s="15" t="inlineStr">
         <is>
           <t>Pregunta si tiene carencias detectadas por analítica antes de recomendar cualquier vitamina, tomar de más tampoco es inocuo.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="74" customHeight="1">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
@@ -1802,62 +2110,62 @@
           <t>El éxito en redes no dice nada sobre si una dieta es segura, muchas eliminan grupos enteros de alimentos con restricciones fuertes que funcionan mal a medio plazo. Antes de opinar, cuéntame en qué consiste y qué objetivo persigues, no es lo mismo bajar de peso que sentirte con más energía. También necesito saber si tomas medicación o tienes alguna enfermedad, porque algunas dietas restrictivas interfieren con tratamientos concretos. Si tienes dudas serias, lo más sensato es consultarlo con tu médico o un nutricionista antes de empezar.</t>
         </is>
       </c>
-      <c r="G29" s="10" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>No apruebes la dieta solo porque tiene muchas visualizaciones ni la descalifiques sin preguntar en qué consiste, valórala con criterio.</t>
         </is>
       </c>
-      <c r="H29" s="10" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>Si el paciente tiene diabetes, problemas renales o toma medicación crónica, deriva a nutricionista o médico antes de dar el visto bueno a cualquier dieta restrictiva.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="74" customHeight="1">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>«¿Es verdad que esta vitamina cura el cansancio de raíz?»</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Ninguna vitamina cura el cansancio si no hay una carencia real detrás.</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>Una vitamina solo mejora el cansancio si ese cansancio viene de una carencia real de esa vitamina, y eso se comprueba con una analítica, no con un anuncio. Si el cansancio tiene otra causa, tomarla no va a cambiar nada.</t>
         </is>
       </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>El cansancio tiene muchas causas posibles, desde el sueño y el estrés hasta problemas de tiroides o carencias de hierro o vitamina D. Una vitamina concreta solo ayuda si el cansancio viene precisamente de esa carencia, y eso se confirma con una analítica, no con un anuncio. Tomarla sin saber la causa puede darte una falsa sensación de hacer algo, mientras el motivo real sigue sin tratarse. Si el cansancio es persistente, lo mejor es que te vea el médico y valore qué hay detrás.</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="G30" s="15" t="inlineStr">
         <is>
           <t>No digas que sí 'por probar no pierdes nada', puede retrasar el diagnóstico de una causa real que sí necesita tratamiento.</t>
         </is>
       </c>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="H30" s="15" t="inlineStr">
         <is>
           <t>Si el cansancio lleva semanas o va acompañado de otros síntomas, deriva al médico en lugar de recomendar solo un suplemento.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="74" customHeight="1">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>La novedad que ha visto en televisión o redes</t>
         </is>
@@ -1882,62 +2190,62 @@
           <t>Ese tipo de productos promete un atajo mágico, pero no hay base real para que un parche haga perder peso por sí solo. El peso corporal depende de la alimentación, el movimiento diario y el descanso, no de pegar algo en la piel. Además, algunos de estos productos no están bien regulados y pueden llevar componentes poco claros en el etiquetado. Si de verdad te interesa perder peso, prefiero orientarte hacia algo con base real que hacia un producto de este tipo.</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>No dejes pasar la venta sin comentario por no discutir, avisar de que es un engaño evita un gasto inútil y una posible decepción.</t>
         </is>
       </c>
-      <c r="H31" s="10" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>Si insiste en comprarlo en otro sitio, aprovecha para ofrecer una alternativa real de acompañamiento, sin sermonear ni repetir el mismo argumento.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="74" customHeight="1">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>«Es que siempre me lo han dado sin receta.»</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Un antibiótico exige receta en cualquier farmacia, no es algo que decida yo.</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>El antibiótico siempre lleva receta, no depende de la farmacia ni de quién atienda. Si tienes síntomas que te preocupan, hoy mismo te puede ver tu médico o el servicio de urgencias.</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
+      <c r="F32" s="14" t="inlineStr">
         <is>
           <t>Entiendo que te venga mal, pero un antibiótico sin receta no se puede vender en ninguna farmacia, es la ley y no depende de mí. Se exige porque un mal uso genera resistencias que después complican el tratamiento a todos. Si tienes fiebre o el malestar va a más, lo mejor es que te vea hoy tu médico de cabecera o urgencias si es fin de semana. Mientras tanto puedo recomendarte algo para aliviar el síntoma, aunque eso no sustituye el diagnóstico.</t>
         </is>
       </c>
-      <c r="G32" s="14" t="inlineStr">
+      <c r="G32" s="15" t="inlineStr">
         <is>
           <t>No insinúes que en otro momento o con otra persona de la farmacia sí se lo darías, porque no es cierto y genera más insistencia.</t>
         </is>
       </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="H32" s="15" t="inlineStr">
         <is>
           <t>Si el paciente dice llevar varios días con fiebre alta o el cuadro empeora, anímale a acudir a urgencias en vez de esperar cita.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="74" customHeight="1">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
@@ -1962,62 +2270,62 @@
           <t>Puede que te haya pasado alguna vez, pero la exigencia de receta para antibióticos es igual en todas las farmacias, no depende del establecimiento. Que en otro sitio lo hicieran de otra forma no cambia lo que corresponde aquí. Existe esa norma porque un antibiótico mal usado pierde eficacia con el tiempo, y eso acaba afectando a todos, no solo a quien lo toma. Si necesitas valorar tus síntomas, pide cita o acude a urgencias si no puede esperar.</t>
         </is>
       </c>
-      <c r="G33" s="10" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>No entres a valorar ni a criticar lo que hizo otra farmacia, céntrate en explicar la norma que aplicas tú.</t>
         </is>
       </c>
-      <c r="H33" s="10" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>Si el paciente insiste en que 'siempre' se lo dan en otro sitio, no lo discutas, repite la norma con calma y ofrece la alternativa de ver al médico.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="74" customHeight="1">
-      <c r="A34" s="11" t="n">
+      <c r="A34" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>«Es el mismo ansiolítico de siempre, solo que perdí la receta.»</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>Sin receta no puedo dispensar ese tipo de medicamento, aunque sea el habitual.</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="14" t="inlineStr">
         <is>
           <t>Los medicamentos con receta que requieren control especial no se pueden dispensar sin ella, aunque sea el tratamiento de toda la vida. Puedes pedir una copia en tu centro de salud, muchas veces la dan el mismo día.</t>
         </is>
       </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>Sé que es incómodo cuando es un tratamiento que ya conoces, pero ese medicamento necesita receta cada vez, porque requiere seguimiento médico continuo. No dudo de que lo tomas habitualmente, es que la ley no permite dispensarlo de otra forma. En muchos centros de salud dan copia de la receta el mismo día si llamas o pides cita de enfermería. Si te quedas sin dosis antes de conseguirla, coméntalo también allí, a veces hay solución más rápida de lo que parece.</t>
         </is>
       </c>
-      <c r="G34" s="14" t="inlineStr">
+      <c r="G34" s="15" t="inlineStr">
         <is>
           <t>No le digas que 'por esta vez' se lo vas a dar, aunque parezca un caso claro, porque abre la puerta a que se repita con otros.</t>
         </is>
       </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H34" s="15" t="inlineStr">
         <is>
           <t>Si el paciente muestra signos de ansiedad importante por quedarse sin el tratamiento, sugiere que llame hoy mismo a su centro de salud en vez de esperar a mañana.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="74" customHeight="1">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
@@ -2042,62 +2350,62 @@
           <t>Entiendo que sea un lío moverse cuando tu padre no puede salir, pero el medicamento va ligado a su receta, no a que tú me digas cuál es o me enseñes la caja vieja. Muchos centros de salud permiten recoger la receta electrónica desde la tarjeta sanitaria de tu padre sin que él tenga que ir en persona. Si tiene cita de seguimiento próxima, también se puede aprovechar para renovarla. En cuanto la tengas, aquí te lo preparo sin ningún problema.</t>
         </is>
       </c>
-      <c r="G35" s="10" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>No te fíes de que 'ya lo conoces' al paciente o a su familia para saltarte la receta, cada dispensación va con su justificante.</t>
         </is>
       </c>
-      <c r="H35" s="10" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>Si es una urgencia real por quedarse sin medicación crónica, orienta a contactar con el centro de salud o el 061 en vez de dispensar sin receta.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="74" customHeight="1">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>«Deme dos cajas grandes, así no tengo que volver en meses.»</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>Te puedo dar la cantidad que indica la receta, ni más ni menos.</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>La cantidad que puedo dispensar es la que marca la receta o el envase habitual para ese tratamiento, no puedo ampliarla a tu gusto. Si necesitas más para más tiempo, eso lo valora tu médico al prescribir.</t>
         </is>
       </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>Entiendo que te vendría bien no volver tan seguido, pero la cantidad que dispensamos va marcada por la receta, no es algo que yo pueda ampliar libremente. Si tu médico cree que necesitas más para más tiempo, puede indicarlo en la próxima receta. Llevar en casa mucha más medicación de la necesaria tampoco es buena idea, sobre todo si caduca o hay que ajustarla según evoluciones. Lo que sí puedo hacer es avisarte con tiempo para que no te quedes sin nada.</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G36" s="15" t="inlineStr">
         <is>
           <t>No cedas a dar cantidad extra solo para evitar una segunda visita, y no lo presentes como un favor personal.</t>
         </is>
       </c>
-      <c r="H36" s="14" t="inlineStr">
+      <c r="H36" s="15" t="inlineStr">
         <is>
           <t>Si el motivo es dificultad real para desplazarse, coméntale la opción de recogida por un familiar o de que su médico ajuste la duración del tratamiento.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="74" customHeight="1">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
@@ -2122,62 +2430,62 @@
           <t>Entiendo que estés harto de escuchar lo mismo, no es mi intención hacerte perder el tiempo. Pero la respuesta no cambia por más veces que se pregunte, porque no depende de mi criterio, sino de una norma igual para todos. Lo que sí puedo hacer es ayudarte con el problema de fondo: si es para conseguir una receta, decirte cómo pedirla más rápido; si es un síntoma que te preocupa, orientarte sobre si conviene ir al médico hoy mismo.</t>
         </is>
       </c>
-      <c r="G37" s="10" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>No te pongas a la defensiva ni respondas con el mismo tono elevado, eso solo alarga la discusión.</t>
         </is>
       </c>
-      <c r="H37" s="10" t="inlineStr">
+      <c r="H37" s="11" t="inlineStr">
         <is>
           <t>Si el paciente sube mucho el tono o hay otras personas esperando, ofrece atenderle aparte un momento para explicarle la alternativa con calma.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="74" customHeight="1">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>«Total, es lo mismo que venden sin receta en el chino de la esquina.»</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>No es lo mismo, y aquí solo puedo dispensar lo que la ley permite.</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>Puede parecer parecido, pero un medicamento con receta pasa por controles que un producto de otro tipo de establecimiento no tiene. Aquí no puedo dispensarlo sin receta, sea cual sea la comparación.</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="F38" s="14" t="inlineStr">
         <is>
           <t>Entiendo que veas parecido en el envase o en el efecto, pero no es lo mismo: un medicamento con receta ha pasado por una evaluación distinta, y se regula así precisamente porque puede tener riesgos si se usa mal. Lo que venden en otro tipo de establecimiento no está sometido a esas mismas garantías, y compararlo no cambia lo que yo puedo dispensar. Si me dices qué buscas conseguir, miro si hay alguna opción legal que se ajuste a lo que necesitas.</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
+      <c r="G38" s="15" t="inlineStr">
         <is>
           <t>No minimices la comparación diciendo 'bueno, tampoco es tan distinto', porque relativiza justo lo que estás intentando explicar.</t>
         </is>
       </c>
-      <c r="H38" s="14" t="inlineStr">
+      <c r="H38" s="15" t="inlineStr">
         <is>
           <t>Si detectas que el paciente ya usa productos de dudoso origen para automedicarse, es buen momento para preguntar con qué fin y ofrecer una alternativa segura.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="74" customHeight="1">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
@@ -2202,62 +2510,62 @@
           <t>El problema no es la dosis, que puede seguir siendo la correcta, sino que la receta ya no es válida porque ha pasado su fecha de vigencia. Eso significa que, formalmente, ya no tengo constancia de que ese tratamiento siga indicado para ti en este momento. Lo más rápido suele ser pedir una renovación en tu centro de salud, muchas veces se puede tramitar sin necesidad de consulta presencial si es un tratamiento crónico ya conocido. En cuanto tengas la receta actualizada, te lo dispenso sin ningún problema.</t>
         </is>
       </c>
-      <c r="G39" s="10" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>No dispenses fiándote de que 'seguro que sigue siendo lo mismo', la validez de la receta no es negociable.</t>
         </is>
       </c>
-      <c r="H39" s="10" t="inlineStr">
+      <c r="H39" s="11" t="inlineStr">
         <is>
           <t>Aprovecha para explicar que renovar la receta antes de que caduque evita este problema la próxima vez.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="74" customHeight="1">
-      <c r="A40" s="11" t="n">
+      <c r="A40" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>Cuando la respuesta es que no</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>«Démelo ya, que luego le traigo la receta, se lo prometo.»</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>No puedo dispensarlo antes de ver la receta, por mucho que la traigas después.</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="14" t="inlineStr">
         <is>
           <t>El orden tiene que ser al revés: primero la receta, luego la dispensación, no puedo hacerlo fiado. Si la consigues hoy, aquí sigo y te lo preparo en el momento.</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
+      <c r="F40" s="14" t="inlineStr">
         <is>
           <t>Entiendo que confíes en que la vas a traer, pero no es una cuestión de confianza personal, es que legalmente la dispensación tiene que ir acompañada de la receta, no venir después. Si la traes hoy más tarde, encantado de dispensarte en ese momento, no hace falta que sea ahora mismo. Si el problema es que no la puedes conseguir hasta mañana, dime qué necesitas exactamente y vemos si hay alguna alternativa sin receta que te sirva mientras tanto.</t>
         </is>
       </c>
-      <c r="G40" s="14" t="inlineStr">
+      <c r="G40" s="15" t="inlineStr">
         <is>
           <t>No aceptes 'fiar' la dispensación aunque el paciente sea conocido de toda la vida, la norma no depende de la confianza.</t>
         </is>
       </c>
-      <c r="H40" s="14" t="inlineStr">
+      <c r="H40" s="15" t="inlineStr">
         <is>
           <t>Si el paciente parece tener verdadera urgencia médica, oriéntale a urgencias en vez de buscarle un atajo en la farmacia.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="74" customHeight="1">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="8" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
@@ -2282,62 +2590,62 @@
           <t>Entiendo las ganas de ir a por todas, pero más dosis de la que necesitas no ayuda más, puede darte mareos o taquicardia y hacer que lo dejes a la primera semana. Funciona mejor ajustar el tratamiento a tu consumo real: cuántos cigarrillos fumas, si el primero es nada más levantarte, si tienes ansiedad fuerte en momentos concretos. Con esos datos te recomiendo la combinación de parche y chicle o comprimido que mejor se adapta. Si quieres, te hago unas preguntas rápidas ahora.</t>
         </is>
       </c>
-      <c r="G41" s="10" t="inlineStr">
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>No le des la presentación de mayor dosis solo porque lo pide con más convicción, la dosis se ajusta al consumo, no a las ganas.</t>
         </is>
       </c>
-      <c r="H41" s="10" t="inlineStr">
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>Si fuma más de veinte cigarrillos al día o el primero es en los primeros cinco minutos tras levantarse, valora derivar a consulta de deshabituación o a su médico.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="74" customHeight="1">
-      <c r="A42" s="11" t="n">
+      <c r="A42" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>«He probado los parches antes y no me hicieron nada.»</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>A veces el parche solo no basta, hay que combinarlo con algo para el momento de ansiedad.</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>El parche da una base de nicotina durante el día, pero no cubre los picos de ansiedad puntual. Combinarlo con un chicle o comprimido para esos momentos suele funcionar mejor que el parche solo.</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
+      <c r="F42" s="14" t="inlineStr">
         <is>
           <t>Que no te funcionara antes no significa que la terapia de sustitución no sirva, puede que faltara ajustar la estrategia. El parche mantiene un nivel de nicotina estable durante el día, pero cuando aparece un antojo fuerte necesitas algo de acción más rápida, como un chicle o comprimido para ese momento. Muchas personas fallan porque usan solo una cosa cuando necesitaban las dos combinadas. Si vuelves a intentarlo, no te desanimes por un primer fallo.</t>
         </is>
       </c>
-      <c r="G42" s="14" t="inlineStr">
+      <c r="G42" s="15" t="inlineStr">
         <is>
           <t>No digas que 'entonces esto tampoco te va a funcionar', porque desanima justo cuando el paciente está dispuesto a intentarlo de nuevo.</t>
         </is>
       </c>
-      <c r="H42" s="14" t="inlineStr">
+      <c r="H42" s="15" t="inlineStr">
         <is>
           <t>Si ha fallado varias veces con distintos métodos, puede ser buen momento para sugerir que su médico valore un tratamiento con receta.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="74" customHeight="1">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
@@ -2362,62 +2670,62 @@
           <t>Que hayas reducido el tabaco está bien, pero si el vapeador sigue teniendo nicotina, el cuerpo sigue enganchado igual, solo cambia la forma de recibirla. Hay menos información a largo plazo sobre el vapeo que sobre el tabaco, así que no lo consideraría un punto de llegada, más bien un paso intermedio. Si el objetivo es dejarlo del todo, podemos plantear una pauta para reducir también la nicotina del vapeador, con parche o chicle de apoyo. Lo importante es no quedarse ahí pensando que ya está resuelto.</t>
         </is>
       </c>
-      <c r="G43" s="10" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>No valores el vapeo como una alternativa sana o equivalente a haberlo dejado, generaría una falsa sensación de logro.</t>
         </is>
       </c>
-      <c r="H43" s="10" t="inlineStr">
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>Si usa vapeadores con nicotina de concentración alta, pregunta la cantidad para poder orientar mejor la pauta de reducción.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="74" customHeight="1">
-      <c r="A44" s="11" t="n">
+      <c r="A44" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>«Me han dicho que hay una pastilla que funciona mejor, ¿me la puede dar usted?»</t>
         </is>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>Ese tratamiento lleva receta, tienes que pedirlo a tu médico para que lo valore.</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>Los tratamientos orales para dejar de fumar de mayor eficacia llevan receta médica, no los puedo dispensar sin ella. Coméntaselo a tu médico, puede valorar si es adecuado para ti.</t>
         </is>
       </c>
-      <c r="F44" s="13" t="inlineStr">
+      <c r="F44" s="14" t="inlineStr">
         <is>
           <t>Existen tratamientos orales que se recetan para dejar de fumar y que en algunos casos funcionan mejor que los parches o chicles solos, pero necesitan receta porque hay que valorar antes tu historial médico y posibles contraindicaciones. Yo no te lo puedo dar sin esa valoración. Te recomiendo pedir cita con tu médico y decirle que quieres dejar de fumar y que te interesa esa opción, así valora si encaja contigo. Mientras tanto, si quieres, empezamos con algo sin receta para ir cogiendo impulso.</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
+      <c r="G44" s="15" t="inlineStr">
         <is>
           <t>No minimices la necesidad de valoración médica diciendo que 'es solo para dejar de fumar', tiene contraindicaciones reales que hay que revisar.</t>
         </is>
       </c>
-      <c r="H44" s="14" t="inlineStr">
+      <c r="H44" s="15" t="inlineStr">
         <is>
           <t>Si el paciente tiene antecedentes cardíacos, psiquiátricos o toma otra medicación, es aún más importante que pase por el médico antes de empezar.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="74" customHeight="1">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="8" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
@@ -2442,62 +2750,62 @@
           <t>Me alegra que quieras dejarlo, es de las mejores cosas que puedes hacer por tu embarazo. Pero no quiero recomendarte nada sin que lo revise tu ginecólogo, porque en el embarazo hay que sopesar con cuidado cualquier producto, incluida la sustitución de nicotina. Hay opciones que en algunos casos se consideran, pero la pauta la marca quien lleva tu seguimiento. Mientras consigues cita, apóyate en estrategias sin fármacos: identificar los momentos de más ganas, tener algo para las manos, pedir apoyo a tu entorno.</t>
         </is>
       </c>
-      <c r="G45" s="10" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>No le des ningún sustitutivo de nicotina 'por probar' sin que lo haya valorado antes su médico, en el embarazo no es terreno para improvisar.</t>
         </is>
       </c>
-      <c r="H45" s="10" t="inlineStr">
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>Si hay mucha ansiedad y dificultad real para esperar a la consulta, anímale a llamar antes a su ginecólogo o matrona en vez de aguantar sola.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="74" customHeight="1">
-      <c r="A46" s="11" t="n">
+      <c r="A46" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>«Llevo dos días sin fumar y no aguanto la ansiedad.»</t>
         </is>
       </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>Los primeros días son los peores, un chicle o comprimido de nicotina te puede aliviar ahora.</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>Los dos o tres primeros días son los más duros porque el cuerpo está pidiendo la nicotina de golpe. Un chicle o comprimido de nicotina para esos picos de ansiedad te puede ayudar bastante ahora mismo.</t>
         </is>
       </c>
-      <c r="F46" s="13" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>Enhorabuena por aguantar dos días, es el tramo más difícil, no significa que vayas mal, es el peor momento y va a mejorar. La ansiedad es el cuerpo reclamando la nicotina de siempre, y baja mucho desde la primera semana. Un chicle o comprimido de nicotina actúa rápido para esos picos, cuando más lo necesitas. También ayuda tener algo para las manos y beber agua ante el antojo. No lo dejes ahora, que es cuando más cerca estás de que cueste menos.</t>
         </is>
       </c>
-      <c r="G46" s="14" t="inlineStr">
+      <c r="G46" s="15" t="inlineStr">
         <is>
           <t>No le quites importancia a la ansiedad diciendo que 'es solo cabeza', el síndrome de abstinencia es real y hay que darle una respuesta práctica.</t>
         </is>
       </c>
-      <c r="H46" s="14" t="inlineStr">
+      <c r="H46" s="15" t="inlineStr">
         <is>
           <t>Si la ansiedad viene con insomnio importante o mucha irritabilidad, coméntaselo también a su médico por si conviene un apoyo adicional.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="74" customHeight="1">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
@@ -2522,62 +2830,62 @@
           <t>Sí se pueden combinar, y para muchas personas funciona mejor que usar un solo formato: el parche mantiene un nivel estable de nicotina durante el día y el chicle o comprimido cubre los momentos de ansiedad más fuerte. Lo importante es no pasarte de la dosis total recomendada entre los dos, así que conviene que te asesoren bien según cuánto fumabas antes. No es peligroso si se usa como está indicado, el riesgo mayor es seguir fumando con el parche puesto, eso sí hay que evitarlo.</t>
         </is>
       </c>
-      <c r="G47" s="10" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>No lo desaconsejes por sistema pensando que 'menos es más seguro', la combinación bien pautada suele dar mejores resultados que un solo formato.</t>
         </is>
       </c>
-      <c r="H47" s="10" t="inlineStr">
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>Explica siempre que no se debe fumar mientras se lleva el parche puesto, ese es el riesgo real, no la combinación en sí.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="74" customHeight="1">
-      <c r="A48" s="11" t="n">
+      <c r="A48" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>«He engordado desde que lo dejé, ¿hay algo para no comer tanto?»</t>
         </is>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>Es habitual coger algo de peso al principio, pero no conviene tratarlo con otro fármaco.</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>Coger algo de peso al dejar de fumar es muy habitual, el cuerpo cambia el metabolismo y muchas veces se sustituye el cigarrillo por picar algo. No recomiendo tratarlo con otro producto encima, mejor ajustar hábitos.</t>
         </is>
       </c>
-      <c r="F48" s="13" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>Es de las cosas más comunes al dejar de fumar, no es que hagas algo mal, es una reacción esperable del cuerpo. El aumento suele venir de sustituir el gesto de fumar por picar entre horas, más que de un cambio en el apetito. Antes de un producto para el peso, que podría interactuar con tu tratamiento, prueba a tener a mano algo para las manos que no sea comida, como agua o fruta. Si el aumento te preocupa, coméntalo con tu médico antes de combinar tratamientos.</t>
         </is>
       </c>
-      <c r="G48" s="14" t="inlineStr">
+      <c r="G48" s="15" t="inlineStr">
         <is>
           <t>No recomiendes un producto para adelgazar o quitar el apetito sin valorar qué está tomando ya para dejar de fumar, podría interactuar.</t>
         </is>
       </c>
-      <c r="H48" s="14" t="inlineStr">
+      <c r="H48" s="15" t="inlineStr">
         <is>
           <t>Si el aumento de peso es mucho o rápido, sugiere revisarlo con su médico junto con el seguimiento de dejar de fumar, no por separado.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="74" customHeight="1">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Dejar de fumar</t>
         </is>
@@ -2602,62 +2910,62 @@
           <t>No todo el mundo necesita tratamiento para dejar de fumar, y con cinco al día puede que lo consigas con fuerza de voluntad. Lo que marca la diferencia no es el número de cigarrillos sino la dependencia: si fumas el primero nada más levantarte, indica más dependencia de la que parece por la cantidad. Si es tu caso, un chicle de nicotina puntual te puede facilitar las cosas. Si no notas gran cosa al dejarlo, prueba primero sin nada y aquí me tienes si hace falta.</t>
         </is>
       </c>
-      <c r="G49" s="10" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>No des por hecho que poco consumo significa poca dependencia, hay que preguntar por el momento del primer cigarrillo, no solo contar unidades.</t>
         </is>
       </c>
-      <c r="H49" s="10" t="inlineStr">
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>Unas pocas preguntas sencillas sobre el momento del primer cigarrillo ayudan a valorar el nivel de dependencia real, más allá del número de cigarrillos.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="74" customHeight="1">
-      <c r="A50" s="11" t="n">
+      <c r="A50" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>«Deme un probiótico bueno, que he oído que van bien para todo.»</t>
         </is>
       </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>Depende de para qué lo necesites, hay cepas distintas según el problema.</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E50" s="14" t="inlineStr">
         <is>
           <t>No todos los probióticos sirven para lo mismo, depende de la cepa y de para qué lo necesites: digestión, después de un antibiótico, molestias intestinales concretas. Cuéntame qué te pasa y te oriento mejor.</t>
         </is>
       </c>
-      <c r="F50" s="13" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
         <is>
           <t>Es verdad que se habla mucho de los probióticos, pero no funcionan todos igual ni sirven 'para todo', cada cepa se ha estudiado para situaciones distintas. Si me cuentas si es por molestias digestivas habituales, por un antibiótico o por mantenimiento, te recomiendo algo más ajustado. Elegir al azar no suele dar mal resultado, pero tampoco aprovechas lo que realmente puede ayudarte. Y si las molestias son persistentes o importantes, conviene que lo valore también tu médico.</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr">
+      <c r="G50" s="15" t="inlineStr">
         <is>
           <t>No entregues 'el probiótico más vendido' sin preguntar el motivo, cada situación se beneficia de una cepa distinta.</t>
         </is>
       </c>
-      <c r="H50" s="14" t="inlineStr">
+      <c r="H50" s="15" t="inlineStr">
         <is>
           <t>Si hay síntomas digestivos persistentes, con sangre o pérdida de peso, es momento de derivar al médico, no de seguir probando complementos.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="74" customHeight="1">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
@@ -2682,62 +2990,62 @@
           <t>No hace falta en todos los casos, pero si sueles notar el estómago revuelto o diarrea con antibióticos, un probiótico durante el tratamiento puede ayudarte. Tómalo separado unas horas del antibiótico, porque si coinciden se pueden neutralizar entre sí. Si nunca has tenido problemas digestivos con antibióticos, no es imprescindible, aunque tampoco hace daño por precaución. Si la diarrea es muy intensa o no mejora, coméntalo con tu médico, no solo con un complemento.</t>
         </is>
       </c>
-      <c r="G51" s="10" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>No digas que hay que tomarlo 'sí o sí' con cualquier antibiótico, no siempre es necesario y generaría un gasto innecesario.</t>
         </is>
       </c>
-      <c r="H51" s="10" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>Recuerda siempre separar la toma del probiótico y el antibiótico unas dos horas para que no pierda efecto.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="74" customHeight="1">
-      <c r="A52" s="11" t="n">
+      <c r="A52" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>«Quiero vitaminas para las defensas, que en el trabajo se contagia todo.»</t>
         </is>
       </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="D52" s="14" t="inlineStr">
         <is>
           <t>Puedo recomendarte algo, pero primero mira si duermes y comes bien, es la base.</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
+      <c r="E52" s="14" t="inlineStr">
         <is>
           <t>Hay complementos que pueden ayudar a sostener el sistema inmunitario, pero antes conviene revisar lo básico: sueño, alimentación variada y estrés, porque sin eso el complemento hace poco. Te recomiendo algo ajustado a tu caso.</t>
         </is>
       </c>
-      <c r="F52" s="13" t="inlineStr">
+      <c r="F52" s="14" t="inlineStr">
         <is>
           <t>Los complementos pueden echar una mano, pero no sustituyen lo básico: dormir bien, comer variado y no acumular estrés hacen más por las defensas que casi cualquier vitamina. Si tu alimentación es irregular o pasas mucho tiempo sin sol, hay opciones que pueden tener sentido para ti. Ninguna te hace inmune a los contagios del trabajo, hay que decirlo claro, pero sí pueden ayudarte a estar en mejores condiciones de fondo. Cuéntame tus hábitos y te recomiendo algo que encaje contigo, en vez de lo primero del lineal.</t>
         </is>
       </c>
-      <c r="G52" s="14" t="inlineStr">
+      <c r="G52" s="15" t="inlineStr">
         <is>
           <t>No prometas que un complemento evita los contagios o refuerza las defensas de forma garantizada, no se puede afirmar eso.</t>
         </is>
       </c>
-      <c r="H52" s="14" t="inlineStr">
+      <c r="H52" s="15" t="inlineStr">
         <is>
           <t>Si hay resfriados o infecciones muy frecuentes y seguidas, sugiere comentarlo con su médico, podría no ser solo cuestión de vitaminas.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="74" customHeight="1">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
@@ -2762,62 +3070,62 @@
           <t>No es cuento, pero tampoco es milagro: el colágeno es un complemento habitual para el cartílago y algunas personas notan mejoría en molestias leves, mientras otras no perciben ningún cambio. No lo puedo asegurar como si fuera un tratamiento con efecto garantizado, hay que probarlo y valorarlo en tu caso. Si lo tomas, dale un margen de varias semanas, el efecto no se nota de un día para otro. Y si el dolor es intenso o limita el movimiento, eso ya es terreno del médico, no de un complemento.</t>
         </is>
       </c>
-      <c r="G53" s="10" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>No lo vendas como una solución segura para el dolor articular, sería prometer un resultado que no se puede garantizar.</t>
         </is>
       </c>
-      <c r="H53" s="10" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>Si hay hinchazón, dolor nocturno o limitación de movimiento importante, deriva al médico antes de centrar todo en el complemento.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="74" customHeight="1">
-      <c r="A54" s="11" t="n">
+      <c r="A54" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>«Mi hijo tiene 4 años, ¿le puedo dar probióticos como a mí?»</t>
         </is>
       </c>
-      <c r="D54" s="13" t="inlineStr">
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>No el mismo que tú, hay presentaciones y dosis pensadas para niños.</t>
         </is>
       </c>
-      <c r="E54" s="13" t="inlineStr">
+      <c r="E54" s="14" t="inlineStr">
         <is>
           <t>Los probióticos para niños llevan una dosis y una cepa pensadas para su edad, no es lo mismo que darle el tuyo en menor cantidad. Te puedo recomendar una presentación pediátrica según lo que necesite.</t>
         </is>
       </c>
-      <c r="F54" s="13" t="inlineStr">
+      <c r="F54" s="14" t="inlineStr">
         <is>
           <t>No le des el mismo producto que tomas tú, aunque sea menos cantidad: las formulaciones infantiles llevan cepas y dosis pensadas para su edad y su sistema digestivo, distinto al de un adulto. Hay presentaciones en gotas o sobres pensadas justo para esto, más fáciles de dar. Si tiene molestias digestivas puntuales, cuéntame cuáles para orientarte mejor. Si son persistentes, con fiebre o afectan a cómo come o duerme, eso lo tiene que ver su pediatra antes de seguir con complementos.</t>
         </is>
       </c>
-      <c r="G54" s="14" t="inlineStr">
+      <c r="G54" s="15" t="inlineStr">
         <is>
           <t>No adaptes a ojo la dosis de un producto de adulto para un niño, no es simplemente 'menos cantidad'.</t>
         </is>
       </c>
-      <c r="H54" s="14" t="inlineStr">
+      <c r="H54" s="15" t="inlineStr">
         <is>
           <t>Ante fiebre, vómitos persistentes o mal estado general en el niño, deriva al pediatra sin demora, no lo trates solo con probióticos.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="74" customHeight="1">
-      <c r="A55" s="7" t="n">
+      <c r="A55" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
@@ -2842,62 +3150,62 @@
           <t>Es una buena pregunta: el omega 3 en dosis altas puede influir en la coagulación, y combinado con tu anticoagulante hay que vigilarlo. No está prohibido siempre, depende de la dosis y de cómo esté controlado tu tratamiento, así que no te lo recomiendo sin consultarlo antes con quien lleva tu anticoagulación. Si quieres más omega 3, suele ser más seguro con la alimentación mientras se confirma, en vez de un complemento concentrado. En cuanto tengas el visto bueno, te ayudo a elegir la dosis.</t>
         </is>
       </c>
-      <c r="G55" s="10" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>No vendas el complemento asegurando que 'es natural, no pasa nada', las interacciones con anticoagulantes son reales aunque el producto sea de origen natural.</t>
         </is>
       </c>
-      <c r="H55" s="10" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Cualquier complemento que pueda afectar a la coagulación merece revisar interacción con el tratamiento antes de venderlo.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="74" customHeight="1">
-      <c r="A56" s="11" t="n">
+      <c r="A56" s="12" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
+      <c r="C56" s="14" t="inlineStr">
         <is>
           <t>«¿Cuál es mejor, el probiótico de sobres o el de cápsulas?»</t>
         </is>
       </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>No es que uno sea mejor, depende de la cepa y de lo que necesites.</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>La forma, sobre o cápsula, es sobre todo una cuestión de comodidad, lo que de verdad importa es la cepa y la cantidad de microorganismos que lleva. Dime para qué lo quieres y miramos cuál se ajusta mejor.</t>
         </is>
       </c>
-      <c r="F56" s="13" t="inlineStr">
+      <c r="F56" s="14" t="inlineStr">
         <is>
           <t>El formato en sí no determina que uno sea mejor, lo que hay que mirar es qué cepas contiene y en qué cantidad, que es lo que influye en el efecto. Los sobres suelen ser más fáciles si te cuesta tragar cápsulas o prefieres disolverlo en agua, pero eso es comodidad, no eficacia. Si me dices para qué lo quieres, molestias digestivas, tras un antibiótico o por mantenimiento, te oriento sobre cuál se ajusta mejor, más allá del formato.</t>
         </is>
       </c>
-      <c r="G56" s="14" t="inlineStr">
+      <c r="G56" s="15" t="inlineStr">
         <is>
           <t>No respondas solo por preferencia personal o por lo que más se vende, la elección depende de la cepa y del motivo, no del formato.</t>
         </is>
       </c>
-      <c r="H56" s="14" t="inlineStr">
+      <c r="H56" s="15" t="inlineStr">
         <is>
           <t>Guarda el envase o el prospecto a mano para poder comparar cepas cuando el paciente pregunte por diferencias entre productos.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="74" customHeight="1">
-      <c r="A57" s="7" t="n">
+      <c r="A57" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
@@ -2922,62 +3230,62 @@
           <t>Que la melatonina no te funcionara no significa que no haya nada más, hay otras plantas con efecto relajante que actúan distinto y a algunas personas les va mejor. Pero antes me interesa saber si tu problema es conciliar el sueño o si te despiertas a media noche y no vuelves a dormir, porque no se trata igual. También conviene mirar tus hábitos antes de dormir: pantallas, horarios, cafeína por la tarde. Si el insomnio lleva meses y te afecta al día a día, coméntaselo también a tu médico.</t>
         </is>
       </c>
-      <c r="G57" s="10" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>No cambies de complemento sin preguntar qué tipo de insomnio tiene, conciliar o mantener el sueño necesitan enfoques distintos.</t>
         </is>
       </c>
-      <c r="H57" s="10" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Insomnio de varios meses de evolución con impacto claro en el día a día merece valoración médica, no una cadena de complementos distintos.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="74" customHeight="1">
-      <c r="A58" s="11" t="n">
+      <c r="A58" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>Complementos y probióticos</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>«¿Me puedo tomar el probiótico a la vez que el antibiótico o mejor separado?»</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>Mejor sepáralos unas dos horas, así el antibiótico no anula el probiótico.</t>
         </is>
       </c>
-      <c r="E58" s="13" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>Si los tomas juntos, el antibiótico puede eliminar buena parte del probiótico antes de que haga efecto. Lo ideal es dejar unas dos horas de diferencia entre uno y otro.</t>
         </is>
       </c>
-      <c r="F58" s="13" t="inlineStr">
+      <c r="F58" s="14" t="inlineStr">
         <is>
           <t>Buena pregunta: si tomas el probiótico justo con el antibiótico, este puede eliminar buena parte de los microorganismos antes de que hagan su función. Lo recomendable es separar las tomas al menos dos horas, por ejemplo el antibiótico con el desayuno y el probiótico a media mañana. Si tomas varias dosis al día, encaja el probiótico en el hueco más alejado de todas. Mantenlo también unos días tras terminar el antibiótico, suele ayudar más si se continúa un poco más.</t>
         </is>
       </c>
-      <c r="G58" s="14" t="inlineStr">
+      <c r="G58" s="15" t="inlineStr">
         <is>
           <t>No digas que da igual el orden o el horario, tomarlos juntos reduce mucho el sentido de dar el probiótico.</t>
         </is>
       </c>
-      <c r="H58" s="14" t="inlineStr">
+      <c r="H58" s="15" t="inlineStr">
         <is>
           <t>Si el paciente tiene varias tomas de antibiótico al día, ayúdale a planificar un horario concreto para encajar el probiótico sin que coincidan.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="74" customHeight="1">
-      <c r="A59" s="7" t="n">
+      <c r="A59" s="8" t="n">
         <v>55</v>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
@@ -3002,62 +3310,62 @@
           <t>Antes de recomendarte nada tengo que verla, una mancha roja puede ser desde una irritación puntual hasta una alergia o algo que necesite diagnóstico médico, y no puedo saberlo solo de oídas. Si al mirarla veo piel irritada sin heridas ni supuración, puedo ofrecerte algo calmante para aliviar la molestia. Si lleva más de unos días, cambia de aspecto o te preocupa, te digo directamente que pases por el médico de cabecera o el dermatólogo.</t>
         </is>
       </c>
-      <c r="G59" s="10" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>Recomendar una crema sin haber mirado la piel, porque puedes tapar o empeorar algo que necesita diagnóstico.</t>
         </is>
       </c>
-      <c r="H59" s="10" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>Cualquier lesión de más de dos o tres semanas, que sangre, cambie de forma o color, se deriva sin dudarlo.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="74" customHeight="1">
-      <c r="A60" s="11" t="n">
+      <c r="A60" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>«¿Este protector solar me vale si tengo la piel muy sensible?»</t>
         </is>
       </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>Sí, este lleva filtros minerales, va bien con pieles sensibles.</t>
         </is>
       </c>
-      <c r="E60" s="13" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>Para piel sensible suelo recomendar los que llevan filtros minerales, dan menos reacciones que algunos filtros químicos. Si nunca lo has usado, pruébalo primero en una zona pequeña de piel.</t>
         </is>
       </c>
-      <c r="F60" s="13" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>Con piel sensible buscamos un protector con filtros minerales, de textura ligera y sin perfume si tiendes a irritarte. No hay un producto que valga para todo el mundo, así que si es la primera vez que usas esta marca te recomiendo probarlo un par de días en la cara interna del brazo antes de aplicarlo en la cara. Y recuerda reaplicarlo cada dos horas si estás al sol, una sola aplicación no dura todo el día.</t>
         </is>
       </c>
-      <c r="G60" s="14" t="inlineStr">
+      <c r="G60" s="15" t="inlineStr">
         <is>
           <t>Decir que un protector no da alergia a nadie, nadie puede prometer eso.</t>
         </is>
       </c>
-      <c r="H60" s="14" t="inlineStr">
+      <c r="H60" s="15" t="inlineStr">
         <is>
           <t>Si la piel sensible viene con rojez constante o granitos, vale la pena preguntar si ya lo ha valorado un dermatólogo.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="74" customHeight="1">
-      <c r="A61" s="7" t="n">
+      <c r="A61" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
@@ -3082,62 +3390,62 @@
           <t>Lo primero es saber la edad del niño, porque no es lo mismo el acné de un adolescente que unos granitos en un bebé, que casi siempre se van solos. Para acné leve en adolescentes hay rutinas de limpieza suave e hidratación que ayudan bastante sin necesitar receta. Si los granos son muchos, duelen, dejan marca o no mejoran en unas semanas, conviene pasar por el dermatólogo, porque hay tratamientos con receta que van más rápido que probar cosas sueltas.</t>
         </is>
       </c>
-      <c r="G61" s="10" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>Tratar igual un brote de acné adolescente que una erupción en un bebé, son cosas distintas.</t>
         </is>
       </c>
-      <c r="H61" s="10" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>Acné con quistes, dolor o marcas que no se van se deriva a dermatología, no se alarga con productos de venta libre.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="74" customHeight="1">
-      <c r="A62" s="11" t="n">
+      <c r="A62" s="12" t="n">
         <v>58</v>
       </c>
-      <c r="B62" s="12" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
         <is>
           <t>«Se me está cayendo mucho el pelo últimamente.»</t>
         </is>
       </c>
-      <c r="D62" s="13" t="inlineStr">
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>¿Desde cuándo notas que se te cae más de lo normal?</t>
         </is>
       </c>
-      <c r="E62" s="13" t="inlineStr">
+      <c r="E62" s="14" t="inlineStr">
         <is>
           <t>La caída puede tener muchas causas, desde estrés o cambio de estación hasta temas de hierro o tiroides. Hay complementos que ayudan a fortalecer, pero si llevas meses así conviene un análisis.</t>
         </is>
       </c>
-      <c r="F62" s="13" t="inlineStr">
+      <c r="F62" s="14" t="inlineStr">
         <is>
           <t>Todos perdemos pelo a diario, así que primero pregunto desde cuándo lo notas y si ha pasado algo antes, un parto, mucho estrés o un cambio de estación, porque en otoño y primavera es habitual que se caiga algo más. Si es algo puntual, hay complementos que ayudan a acompañar el ciclo del pelo. Si llevas más de tres meses con caída notable o ves entradas o calvas, te recomiendo pasar por el médico para descartar hierro, tiroides o algo hormonal.</t>
         </is>
       </c>
-      <c r="G62" s="14" t="inlineStr">
+      <c r="G62" s="15" t="inlineStr">
         <is>
           <t>Vender el complemento como solución sin preguntar antes cuánto tiempo lleva ni si hay una causa clara.</t>
         </is>
       </c>
-      <c r="H62" s="14" t="inlineStr">
+      <c r="H62" s="15" t="inlineStr">
         <is>
           <t>Caída brusca en placas o mechones se deriva siempre a dermatología, no es una caída difusa normal.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="74" customHeight="1">
-      <c r="A63" s="7" t="n">
+      <c r="A63" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
@@ -3162,62 +3470,62 @@
           <t>Antes de recomendarte una en concreto me gusta saber si tu piel es seca o mixta, si te preocupan las líneas de expresión o más bien la flacidez, y si ya usas retinol. El ácido hialurónico hidrata y rellena superficialmente, los retinoides suaves ayudan a renovar la piel pero pueden dar sequedad al principio, y los péptidos se llevan mejor con pieles sensibles. Lo importante es usarla de forma constante y con protector solar por el día, sin eso el efecto se pierde.</t>
         </is>
       </c>
-      <c r="G63" s="10" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>Prometer que una crema elimina las arrugas, mejor hablar de mejorar el aspecto o cuidar la piel.</t>
         </is>
       </c>
-      <c r="H63" s="10" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>Si empieza con retinol por primera vez, avisar de que puede dar algo de irritación las primeras semanas y que vaya poco a poco.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="74" customHeight="1">
-      <c r="A64" s="11" t="n">
+      <c r="A64" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B64" s="12" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
       </c>
-      <c r="C64" s="13" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
         <is>
           <t>«Llevo días con la piel seca y tirante, ¿es por el aire acondicionado?»</t>
         </is>
       </c>
-      <c r="D64" s="13" t="inlineStr">
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>Puede ser, el aire seco reseca mucho la piel, prueba una crema más nutritiva.</t>
         </is>
       </c>
-      <c r="E64" s="13" t="inlineStr">
+      <c r="E64" s="14" t="inlineStr">
         <is>
           <t>El aire acondicionado y la calefacción resecan bastante la piel, sí. Te recomiendo una crema con más contenido graso y beber agua a lo largo del día. Si además pica mucho, dímelo.</t>
         </is>
       </c>
-      <c r="F64" s="13" t="inlineStr">
+      <c r="F64" s="14" t="inlineStr">
         <is>
           <t>El aire acondicionado y la calefacción son de las causas más frecuentes de piel tirante, porque bajan la humedad ambiente y la piel pierde agua más rápido. Lo primero es cambiar a una crema algo más nutritiva, sobre todo donde más lo notas. También ayuda beber agua durante el día, no solo cuando tienes sed, y evitar duchas muy calientes. Si en una semana no mejora, o pica bastante o ves la piel agrietada, mejor que le echemos otro vistazo.</t>
         </is>
       </c>
-      <c r="G64" s="14" t="inlineStr">
+      <c r="G64" s="15" t="inlineStr">
         <is>
           <t>Quitarle importancia sin más, la sequedad mantenida puede acabar en dermatitis si no se cuida.</t>
         </is>
       </c>
-      <c r="H64" s="14" t="inlineStr">
+      <c r="H64" s="15" t="inlineStr">
         <is>
           <t>Picor intenso, grietas o piel que se agrieta y sangra es motivo de consulta, no solo de crema.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="74" customHeight="1">
-      <c r="A65" s="7" t="n">
+      <c r="A65" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
@@ -3242,62 +3550,62 @@
           <t>Entiendo que quieras solucionarlo rápido, pero las lesiones de espalda son de las que más se confunden entre sí, desde hongos hasta dermatitis o manchas de sol, y cada una necesita un tratamiento distinto. Si tratas un hongo con algo que no es antifúngico, o al revés, puedes retrasar la mejora sin darte cuenta. Prefiero que pase primero por el médico o el dermatólogo para tener un diagnóstico claro, y luego yo te ayudo con el tratamiento y te explico cómo aplicarlo.</t>
         </is>
       </c>
-      <c r="G65" s="10" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>Vender un antifúngico a ciegas solo porque el paciente lo pide, si no es hongo no va a mejorar.</t>
         </is>
       </c>
-      <c r="H65" s="10" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Las lesiones que no se ven bien a simple vista o en zonas que el paciente no puede enseñar cómodamente, siempre se derivan.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="74" customHeight="1">
-      <c r="A66" s="11" t="n">
+      <c r="A66" s="12" t="n">
         <v>62</v>
       </c>
-      <c r="B66" s="12" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>«Tengo la piel del bebé con rojeces en el pañal, ¿qué le pongo?»</t>
         </is>
       </c>
-      <c r="D66" s="13" t="inlineStr">
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>Para el pañal van bien las pastas con óxido de zinc, cambia el pañal a menudo.</t>
         </is>
       </c>
-      <c r="E66" s="13" t="inlineStr">
+      <c r="E66" s="14" t="inlineStr">
         <is>
           <t>Lo habitual es una pasta al agua con óxido de zinc en cada cambio, y dejar que la piel respire un rato sin pañal. Si no mejora en dos o tres días, que lo vea el pediatra.</t>
         </is>
       </c>
-      <c r="F66" s="13" t="inlineStr">
+      <c r="F66" s="14" t="inlineStr">
         <is>
           <t>El eritema del pañal casi siempre se debe a la humedad y el roce, así que lo primero es cambiar el pañal con más frecuencia y limpiar con agua tibia en vez de toallitas si la piel ya está irritada. Después de cada cambio conviene aplicar una pasta al agua con óxido de zinc, que protege la piel, y dejar un rato al bebé sin pañal si puedes. Si en dos días no mejora o aparecen ampollas o pus, hay que descartar infección y eso lo valora el pediatra.</t>
         </is>
       </c>
-      <c r="G66" s="14" t="inlineStr">
+      <c r="G66" s="15" t="inlineStr">
         <is>
           <t>Minimizar una rojez que lleva días o que tiene aspecto de infectada, en bebés se deriva pronto.</t>
         </is>
       </c>
-      <c r="H66" s="14" t="inlineStr">
+      <c r="H66" s="15" t="inlineStr">
         <is>
           <t>Preguntar siempre si ya ha probado alguna crema, para no repetir lo mismo que no ha funcionado.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="74" customHeight="1">
-      <c r="A67" s="7" t="n">
+      <c r="A67" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="B67" s="8" t="inlineStr">
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>Dermofarmacia y consulta de piel</t>
         </is>
@@ -3322,62 +3630,62 @@
           <t>Sí, es posible que aparezcan lunares nuevos en cualquier momento de la vida, no es solo cosa de la infancia. Dicho esto, un lunar nuevo en un adulto, sobre todo si aparece de golpe, tiene bordes irregulares, colores distintos dentro de la misma mancha o crece rápido, es justo lo que un dermatólogo quiere revisar cuanto antes. No te puedo decir si el tuyo es motivo de preocupación sin verlo con las herramientas adecuadas, así que te recomiendo pedir cita, sobre todo si tienes muchos lunares o antecedentes familiares.</t>
         </is>
       </c>
-      <c r="G67" s="10" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>Decir seguro que no es nada sin haberlo visto, no es una valoración que se pueda hacer así.</t>
         </is>
       </c>
-      <c r="H67" s="10" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>La revisión dermatológica anual es buena práctica si hay muchos lunares o piel muy clara, coméntaselo aunque no lo pregunte.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="74" customHeight="1">
-      <c r="A68" s="11" t="n">
+      <c r="A68" s="12" t="n">
         <v>64</v>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
+      <c r="C68" s="14" t="inlineStr">
         <is>
           <t>«En internet lo he visto a mitad de precio.»</t>
         </is>
       </c>
-      <c r="D68" s="13" t="inlineStr">
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>Puede ser, aquí llevas el consejo de que es el producto adecuado para ti.</t>
         </is>
       </c>
-      <c r="E68" s="13" t="inlineStr">
+      <c r="E68" s="14" t="inlineStr">
         <is>
           <t>Es posible que en internet salga más barato, cada canal tiene sus costes. Lo que te doy aquí es que compruebo que es lo que necesitas y cómo usarlo bien.</t>
         </is>
       </c>
-      <c r="F68" s="13" t="inlineStr">
+      <c r="F68" s="14" t="inlineStr">
         <is>
           <t>Puede que sí, en internet hay mucha variedad de precios y no siempre sabes de dónde viene el producto ni en qué condiciones ha llegado. Aquí lo que tienes es que antes de dártelo compruebo que es el producto adecuado para tu caso, te explico cómo usarlo y qué esperar, y si algo no va bien puedes volver y lo resolvemos en el momento. Si al final decides comprarlo online, no pasa nada, pero si tienes dudas de si es lo que necesitas, para eso estamos.</t>
         </is>
       </c>
-      <c r="G68" s="14" t="inlineStr">
+      <c r="G68" s="15" t="inlineStr">
         <is>
           <t>Ponerse a la defensiva o hablar mal de las tiendas online, suena a vendedor incómodo.</t>
         </is>
       </c>
-      <c r="H68" s="14" t="inlineStr">
+      <c r="H68" s="15" t="inlineStr">
         <is>
           <t>Si el producto es de uso delicado, como algo dermatológico o para niños, insistir en el valor del consejo sin sonar a excusa de precio.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="74" customHeight="1">
-      <c r="A69" s="7" t="n">
+      <c r="A69" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B69" s="7" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
@@ -3402,62 +3710,62 @@
           <t>En farmacia el precio de muchos productos, sobre todo medicamentos, está fijado y no lo decidimos nosotros libremente. Lo que sí puedo decirte es qué compras además del producto: alguien que revisa que no interacciona con lo que ya tomas, que te explica cómo y cuándo usarlo, y que está aquí si algo va mal después. En otros establecimientos compras solo el producto, sin ese acompañamiento, y en el caso de medicamentos, muchas veces ni siquiera deberían venderse fuera de farmacia.</t>
         </is>
       </c>
-      <c r="G69" s="10" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>Criticar directamente al otro establecimiento, mejor centrarse en lo que aporta la farmacia.</t>
         </is>
       </c>
-      <c r="H69" s="10" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>Si el producto en cuestión no debería venderse fuera de farmacia, decirlo con naturalidad, no como reproche.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="74" customHeight="1">
-      <c r="A70" s="11" t="n">
+      <c r="A70" s="12" t="n">
         <v>66</v>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C70" s="14" t="inlineStr">
         <is>
           <t>«Me han dicho que esta crema y la de la marca blanca son iguales.»</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>Pueden compartir algún ingrediente, pero la fórmula completa no siempre es la misma.</t>
         </is>
       </c>
-      <c r="E70" s="13" t="inlineStr">
+      <c r="E70" s="14" t="inlineStr">
         <is>
           <t>A veces comparten el principio activo principal, pero la concentración, los excipientes o la textura pueden variar bastante. Si quieres, miramos juntos la composición de las dos.</t>
         </is>
       </c>
-      <c r="F70" s="13" t="inlineStr">
+      <c r="F70" s="14" t="inlineStr">
         <is>
           <t>Puede que compartan el ingrediente que más se anuncia, pero una crema no es solo ese ingrediente, también importa la concentración, cómo está formulada para que penetre bien, qué otros componentes lleva y cómo se conserva. Dos productos pueden parecerse en el papel y comportarse distinto en la piel. Si te interesa, miramos juntos el etiquetado de las dos y te explico las diferencias reales que veo, así decides con información y no solo por el precio.</t>
         </is>
       </c>
-      <c r="G70" s="14" t="inlineStr">
+      <c r="G70" s="15" t="inlineStr">
         <is>
           <t>Afirmar sin comprobarlo que son iguales o que son distintas, mejor mirar la composición antes de opinar.</t>
         </is>
       </c>
-      <c r="H70" s="14" t="inlineStr">
+      <c r="H70" s="15" t="inlineStr">
         <is>
           <t>Si el paciente tiene piel sensible o un problema concreto, el cambio de fórmula sí puede notarse aunque el activo principal coincida.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="74" customHeight="1">
-      <c r="A71" s="7" t="n">
+      <c r="A71" s="8" t="n">
         <v>67</v>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
@@ -3482,62 +3790,62 @@
           <t>Sin problema, tómate el tiempo que quieras, no tienes que decidir aquí mismo. Mientras comparas, aprovecho para comentarte cualquier cosa que creas que te puede ayudar a decidir, como si es apto para tu caso concreto o si hay una alternativa que se ajuste mejor a lo que buscas. Decidas lo que decidas, la idea es que salgas de aquí con la información clara, no que te sientas presionado a comprar en el momento.</t>
         </is>
       </c>
-      <c r="G71" s="10" t="inlineStr">
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>Insistir o meter prisa para que compre ya, genera el efecto contrario.</t>
         </is>
       </c>
-      <c r="H71" s="10" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>Aprovechar el momento para dar un dato útil, como cómo se usa o cuánto dura, suele pesar más que el precio en la decisión final.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="74" customHeight="1">
-      <c r="A72" s="11" t="n">
+      <c r="A72" s="12" t="n">
         <v>68</v>
       </c>
-      <c r="B72" s="12" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
       </c>
-      <c r="C72" s="13" t="inlineStr">
+      <c r="C72" s="14" t="inlineStr">
         <is>
           <t>«¿Me hacéis descuento si compro varias unidades?»</t>
         </is>
       </c>
-      <c r="D72" s="13" t="inlineStr">
+      <c r="D72" s="14" t="inlineStr">
         <is>
           <t>En medicamentos no podemos, en parafarmacia depende del producto, te lo miro.</t>
         </is>
       </c>
-      <c r="E72" s="13" t="inlineStr">
+      <c r="E72" s="14" t="inlineStr">
         <is>
           <t>En medicamentos el precio está fijado y no se puede tocar. En productos de parafarmacia a veces sí hay packs o promociones, te miro si aplica a este.</t>
         </is>
       </c>
-      <c r="F72" s="13" t="inlineStr">
+      <c r="F72" s="14" t="inlineStr">
         <is>
           <t>Depende de qué sea. Si es un medicamento, el precio viene fijado y no podemos aplicar descuentos aunque compres varias cajas, es así para todas las farmacias por igual. Si es un producto de parafarmacia, como cosmética o complementos, a veces sí tenemos packs, formatos ahorro o promociones puntuales, así que déjame mirarlo en el sistema antes de decirte que no. Si no hay nada ahora mismo, te aviso si entra alguna promoción más adelante.</t>
         </is>
       </c>
-      <c r="G72" s="14" t="inlineStr">
+      <c r="G72" s="15" t="inlineStr">
         <is>
           <t>Decir que no se hacen descuentos sin comprobar si el producto concreto tiene alguna promoción activa.</t>
         </is>
       </c>
-      <c r="H72" s="14" t="inlineStr">
+      <c r="H72" s="15" t="inlineStr">
         <is>
           <t>Diferenciar siempre medicamento de parafarmacia al hablar de precio, son normativas distintas.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="74" customHeight="1">
-      <c r="A73" s="7" t="n">
+      <c r="A73" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
@@ -3562,62 +3870,62 @@
           <t>Depende del tipo de producto. Si es un medicamento, el precio está regulado y tiene que ser el mismo en cualquier farmacia de España, así que si hay diferencia ahí vale la pena revisarlo. Si es un producto de parafarmacia, cada farmacia decide su margen según sus costes, así que puede haber diferencias de precio de un pueblo a otro, igual que pasa con cualquier otro comercio. No es que uno cobre de más, es que no hay un precio único fijado para ese tipo de producto.</t>
         </is>
       </c>
-      <c r="G73" s="10" t="inlineStr">
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>Justificarse de más o sonar como si se sintiera acusado, es una diferencia normal del sistema.</t>
         </is>
       </c>
-      <c r="H73" s="10" t="inlineStr">
+      <c r="H73" s="11" t="inlineStr">
         <is>
           <t>Si el paciente insiste mucho, ofrecerle mirar si hay una alternativa de precio más ajustado dentro de la misma categoría.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="74" customHeight="1">
-      <c r="A74" s="11" t="n">
+      <c r="A74" s="12" t="n">
         <v>70</v>
       </c>
-      <c r="B74" s="12" t="inlineStr">
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
         <is>
           <t>«¿Vale la pena pagar la marca o me sirve la genérica?»</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D74" s="14" t="inlineStr">
         <is>
           <t>Para el mismo principio activo, el genérico tiene la misma eficacia demostrada.</t>
         </is>
       </c>
-      <c r="E74" s="13" t="inlineStr">
+      <c r="E74" s="14" t="inlineStr">
         <is>
           <t>Si hablamos de medicamentos, el genérico lleva el mismo principio activo y pasa los mismos controles, la diferencia suele ser el precio. En cosmética es distinto, ahí sí varía la fórmula completa.</t>
         </is>
       </c>
-      <c r="F74" s="13" t="inlineStr">
+      <c r="F74" s="14" t="inlineStr">
         <is>
           <t>Depende de si hablamos de un medicamento o de cosmética. En medicamentos, el genérico demuestra la misma eficacia y seguridad que la marca original antes de venderse, la diferencia suele estar en el precio y a veces en algún excipiente, que solo importa si tienes alguna alergia concreta. En cosmética el concepto de genérico no existe igual, cada marca tiene su propia fórmula, así que ahí sí puede haber diferencias reales en textura o resultado, y merece la pena hablar de tu caso concreto antes de decidir.</t>
         </is>
       </c>
-      <c r="G74" s="14" t="inlineStr">
+      <c r="G74" s="15" t="inlineStr">
         <is>
           <t>Meter en el mismo saco medicamentos y cosmética, son situaciones distintas y hay que explicarlo así.</t>
         </is>
       </c>
-      <c r="H74" s="14" t="inlineStr">
+      <c r="H74" s="15" t="inlineStr">
         <is>
           <t>Si hay antecedentes de alergia a algún excipiente, revisar el prospecto del genérico antes de sustituir.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="74" customHeight="1">
-      <c r="A75" s="7" t="n">
+      <c r="A75" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
@@ -3642,62 +3950,62 @@
           <t>Totalmente respetable, si no hay prisa y prefieres esperar unos días para ahorrarte algo, es tu decisión y no hay ningún problema. Lo único que te diría es que valores si es algo que necesitas empezar a usar ya, porque unos días de retraso a veces sí importan, por ejemplo si es para una molestia que ya tienes o antes de un viaje. Si decides esperar, cuando te llegue y tengas dudas de cómo usarlo, puedes venir igualmente y te lo explico sin problema.</t>
         </is>
       </c>
-      <c r="G75" s="10" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>Sonar molesto porque decide comprarlo fuera, la decisión es del paciente y no hay que forzarla.</t>
         </is>
       </c>
-      <c r="H75" s="10" t="inlineStr">
+      <c r="H75" s="11" t="inlineStr">
         <is>
           <t>Si el motivo de la compra es urgente, como dolor, fiebre o un viaje inminente, remarcarlo con suavidad puede cambiar la decisión.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="74" customHeight="1">
-      <c r="A76" s="11" t="n">
+      <c r="A76" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>El precio y la comparación con internet</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>«¿Por qué el mismo complemento cambia tanto de precio según la farmacia?»</t>
         </is>
       </c>
-      <c r="D76" s="13" t="inlineStr">
+      <c r="D76" s="14" t="inlineStr">
         <is>
           <t>Los complementos no tienen precio fijado, cada farmacia pone el suyo.</t>
         </is>
       </c>
-      <c r="E76" s="13" t="inlineStr">
+      <c r="E76" s="14" t="inlineStr">
         <is>
           <t>A diferencia de los medicamentos, los complementos alimenticios no tienen un precio regulado, cada farmacia lo fija libremente. Por eso puedes ver diferencias de una a otra.</t>
         </is>
       </c>
-      <c r="F76" s="13" t="inlineStr">
+      <c r="F76" s="14" t="inlineStr">
         <is>
           <t>Los complementos son parafarmacia, no medicamentos, así que no tienen un precio único fijado por ley como muchos fármacos. Cada farmacia calcula su precio según lo que le cuesta el producto y su política comercial, por eso el mismo complemento puede ser más caro o más barato de una farmacia a otra. Lo que sí te garantizo es que el producto está bien conservado y que si tienes dudas sobre si te conviene o cómo combinarlo con otra cosa, te lo resuelvo antes de que te lo lleves.</t>
         </is>
       </c>
-      <c r="G76" s="14" t="inlineStr">
+      <c r="G76" s="15" t="inlineStr">
         <is>
           <t>Dar a entender que el precio es lo que es sin explicar por qué varía, genera desconfianza.</t>
         </is>
       </c>
-      <c r="H76" s="14" t="inlineStr">
+      <c r="H76" s="15" t="inlineStr">
         <is>
           <t>Aprovechar para preguntar qué otros medicamentos toma, algunos complementos interaccionan y ahí está el valor real del consejo.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="74" customHeight="1">
-      <c r="A77" s="7" t="n">
+      <c r="A77" s="8" t="n">
         <v>73</v>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
@@ -3722,62 +4030,62 @@
           <t>Ahora mismo no tengo existencias de esa marca, pero puedo hacer el pedido hoy mismo y suele llegar mañana a primera hora, así que si puedes esperar un día no hay problema. Si te preocupa quedarte sin ella hoy, miro en el sistema si hay otro medicamento con el mismo principio activo y la misma dosis que te pueda servir mientras tanto, y te lo explico bien para que no haya confusión con el envase. Nunca vas a quedarte sin tratamiento por esto, siempre hay una solución.</t>
         </is>
       </c>
-      <c r="G77" s="10" t="inlineStr">
+      <c r="G77" s="11" t="inlineStr">
         <is>
           <t>Decir simplemente que no tenéis, sin ofrecer alternativa ni plazo, genera alarma innecesaria en tratamientos crónicos.</t>
         </is>
       </c>
-      <c r="H77" s="10" t="inlineStr">
+      <c r="H77" s="11" t="inlineStr">
         <is>
           <t>En medicación crónica, comprobar siempre si hay equivalente antes de mandar al paciente a otra farmacia.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="74" customHeight="1">
-      <c r="A78" s="11" t="n">
+      <c r="A78" s="12" t="n">
         <v>74</v>
       </c>
-      <c r="B78" s="12" t="inlineStr">
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>«Es la tercera farmacia a la que vengo y en ninguna lo tenéis.»</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D78" s="14" t="inlineStr">
         <is>
           <t>Lo siento, hay un problema de suministro general, te lo encargo ya.</t>
         </is>
       </c>
-      <c r="E78" s="13" t="inlineStr">
+      <c r="E78" s="14" t="inlineStr">
         <is>
           <t>Lo sé, es un desabastecimiento que afecta a varias farmacias, no es solo aquí. Te lo pido ahora y en cuanto entre te aviso.</t>
         </is>
       </c>
-      <c r="F78" s="13" t="inlineStr">
+      <c r="F78" s="14" t="inlineStr">
         <is>
           <t>Entiendo la frustración, y no es nada personal de esta farmacia, hay un problema de suministro con ese medicamento que está afectando a bastantes farmacias de la zona, así que es probable que en otras te digan lo mismo. Puedo pedirlo ya mismo y, si el laboratorio avisa de cuándo vuelve a haber stock, te llamo en cuanto llegue para que no tengas que estar viniendo a preguntar. Mientras tanto, si necesitas seguir el tratamiento sin interrupción, miramos juntos si hay una alternativa con el mismo principio activo disponible.</t>
         </is>
       </c>
-      <c r="G78" s="14" t="inlineStr">
+      <c r="G78" s="15" t="inlineStr">
         <is>
           <t>Quitarle importancia a la molestia del paciente, ha perdido tiempo yendo a varios sitios y hay que reconocerlo.</t>
         </is>
       </c>
-      <c r="H78" s="14" t="inlineStr">
+      <c r="H78" s="15" t="inlineStr">
         <is>
           <t>Apuntar el teléfono del paciente para avisar en cuanto llegue evita que vuelva varias veces en balde.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="74" customHeight="1">
-      <c r="A79" s="7" t="n">
+      <c r="A79" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
@@ -3802,62 +4110,62 @@
           <t>El pedido lo hacemos hoy con el almacén y en condiciones normales llega mañana por la mañana, aunque algún caso puntual tarda un poco más si es un producto especial o viene del laboratorio. Para que no tengas que venir a preguntar cada día, apunto tu teléfono y en cuanto llegue te aviso por mensaje o llamada, tú eliges. Si por lo que sea se retrasa más de lo normal, también te lo comunico para que no te quedes esperando sin saber nada.</t>
         </is>
       </c>
-      <c r="G79" s="10" t="inlineStr">
+      <c r="G79" s="11" t="inlineStr">
         <is>
           <t>Dar un plazo si no se está seguro, mejor decir normalmente y comprometerse a avisar que prometer un día exacto.</t>
         </is>
       </c>
-      <c r="H79" s="10" t="inlineStr">
+      <c r="H79" s="11" t="inlineStr">
         <is>
           <t>Confirmar siempre un teléfono de contacto al hacer el encargo, ahorra visitas innecesarias a ambas partes.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="74" customHeight="1">
-      <c r="A80" s="11" t="n">
+      <c r="A80" s="12" t="n">
         <v>76</v>
       </c>
-      <c r="B80" s="12" t="inlineStr">
+      <c r="B80" s="13" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
         <is>
           <t>«Necesito esto para hoy, no puedo esperar a mañana.»</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D80" s="14" t="inlineStr">
         <is>
           <t>Entiendo la urgencia, déjame ver si otra farmacia cercana lo tiene ahora.</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>Si es urgente, te lo miro en el sistema de farmacias cercanas a ver si alguna lo tiene hoy. Si no, valoramos juntos si hay una alternativa válida.</t>
         </is>
       </c>
-      <c r="F80" s="13" t="inlineStr">
+      <c r="F80" s="14" t="inlineStr">
         <is>
           <t>Si realmente no puede esperar, lo primero que hago es consultar si alguna farmacia cercana tiene stock ahora mismo, muchas veces se puede localizar y resolverlo el mismo día. Si ninguna lo tiene, miramos si existe otro medicamento con el mismo principio activo que pueda cubrirte hoy, o si por las características del tratamiento es seguro esperar hasta mañana sin que pase nada. Lo que no quiero es que salgas de aquí sin ninguna solución, así que vamos a resolverlo entre los dos.</t>
         </is>
       </c>
-      <c r="G80" s="14" t="inlineStr">
+      <c r="G80" s="15" t="inlineStr">
         <is>
           <t>Restar urgencia al paciente sin comprobar antes si de verdad puede esperar según el tratamiento.</t>
         </is>
       </c>
-      <c r="H80" s="14" t="inlineStr">
+      <c r="H80" s="15" t="inlineStr">
         <is>
           <t>Si es un tratamiento donde saltarse una toma sí importa, como los anticoagulantes, priorizar buscar en otra farmacia antes que encargar.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="74" customHeight="1">
-      <c r="A81" s="7" t="n">
+      <c r="A81" s="8" t="n">
         <v>77</v>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
@@ -3882,62 +4190,62 @@
           <t>Es una situación bastante frecuente últimamente con ciertos medicamentos, y normalmente viene de problemas en la producción del laboratorio o en la distribución, cosas fuera del control de la farmacia. Cuando hay desabastecimiento, todas las farmacias del país lo notan a la vez, no es que aquí no queramos tenerlo. Lo que sí hacemos es pedirlo en cuanto el sistema indica disponibilidad, y mientras tanto valorar contigo si existe una alternativa con el mismo principio activo que puedas usar sin perder continuidad en el tratamiento.</t>
         </is>
       </c>
-      <c r="G81" s="10" t="inlineStr">
+      <c r="G81" s="11" t="inlineStr">
         <is>
           <t>Sonar como si te desentendieras del problema, mejor mostrar que se está haciendo algo activamente.</t>
         </is>
       </c>
-      <c r="H81" s="10" t="inlineStr">
+      <c r="H81" s="11" t="inlineStr">
         <is>
           <t>Si el desabastecimiento es prolongado, merece la pena consultar con el médico si conviene cambiar de tratamiento de forma más estable.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="74" customHeight="1">
-      <c r="A82" s="11" t="n">
+      <c r="A82" s="12" t="n">
         <v>78</v>
       </c>
-      <c r="B82" s="12" t="inlineStr">
+      <c r="B82" s="13" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>«¿Me lo podéis guardar para que no se agote cuando llegue?»</t>
         </is>
       </c>
-      <c r="D82" s="13" t="inlineStr">
+      <c r="D82" s="14" t="inlineStr">
         <is>
           <t>Claro, te lo aparto en cuanto entre y te aviso.</t>
         </is>
       </c>
-      <c r="E82" s="13" t="inlineStr">
+      <c r="E82" s="14" t="inlineStr">
         <is>
           <t>Sin problema, apunto tu pedido y en cuanto llegue lo aparto a tu nombre. Te aviso para que vengas cuando puedas.</t>
         </is>
       </c>
-      <c r="F82" s="13" t="inlineStr">
+      <c r="F82" s="14" t="inlineStr">
         <is>
           <t>Por supuesto, es justo para eso que hacemos el encargo, apunto tu nombre y tu teléfono junto al pedido para que en cuanto llegue la mercancía la reserve para ti antes de ponerla en el mostrador. Así te evitas venir varios días seguidos a comprobar si ha llegado y encontrarte con que se ha agotado. En cuanto lo tenga aquí, te aviso y lo tienes guardado el tiempo que necesites para venir a recogerlo.</t>
         </is>
       </c>
-      <c r="G82" s="14" t="inlineStr">
+      <c r="G82" s="15" t="inlineStr">
         <is>
           <t>Olvidar apuntar el nombre y el contacto, es lo que evita que el paciente sienta que tiene que estar pendiente él solo.</t>
         </is>
       </c>
-      <c r="H82" s="14" t="inlineStr">
+      <c r="H82" s="15" t="inlineStr">
         <is>
           <t>Si son varias unidades o un tratamiento largo, aclarar si se factura al recogerlo o si se paga por adelantado, según la política de la farmacia.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="74" customHeight="1">
-      <c r="A83" s="7" t="n">
+      <c r="A83" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B83" s="7" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
@@ -3962,62 +4270,62 @@
           <t>Es posible que exista una alternativa válida, pero antes de ofrecértela necesito comprobar que tiene el mismo principio activo, la misma dosis y que no hay diferencia relevante para tu caso, por ejemplo si tomas otra medicación que pueda interaccionar de forma distinta. Dame un momento para mirarlo con calma en el sistema. Si encuentro una opción segura, te la explico bien, y si no la hay, valoramos si puedes esperar al encargo o si conviene consultar con el médico una alternativa distinta.</t>
         </is>
       </c>
-      <c r="G83" s="10" t="inlineStr">
+      <c r="G83" s="11" t="inlineStr">
         <is>
           <t>Ofrecer un sustituto a la ligera sin comprobar dosis ni interacciones solo por salir del paso.</t>
         </is>
       </c>
-      <c r="H83" s="10" t="inlineStr">
+      <c r="H83" s="11" t="inlineStr">
         <is>
           <t>Ante cualquier duda sobre la equivalencia real, mejor llamar al médico o a farmacia hospitalaria que arriesgar.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="74" customHeight="1">
-      <c r="A84" s="11" t="n">
+      <c r="A84" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="B84" s="12" t="inlineStr">
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
       </c>
-      <c r="C84" s="13" t="inlineStr">
+      <c r="C84" s="14" t="inlineStr">
         <is>
           <t>«Vaya faena, tenía que empezar el tratamiento ya.»</t>
         </is>
       </c>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="D84" s="14" t="inlineStr">
         <is>
           <t>Lo entiendo, vamos a ver ahora mismo cómo resolverlo sin que lo pierdas.</t>
         </is>
       </c>
-      <c r="E84" s="13" t="inlineStr">
+      <c r="E84" s="14" t="inlineStr">
         <is>
           <t>Entiendo la urgencia. Miro si alguna farmacia cercana lo tiene o si existe una alternativa que puedas empezar hoy, y seguimos con el encargo en paralelo.</t>
         </is>
       </c>
-      <c r="F84" s="13" t="inlineStr">
+      <c r="F84" s="14" t="inlineStr">
         <is>
           <t>Lo entiendo perfectamente, y por eso no nos quedamos solo con pedirlo y esperar. Primero miro si alguna farmacia de la zona tiene stock ahora, porque a veces se resuelve en la misma mañana. Si no lo hay cerca, buscamos si existe una alternativa con el mismo principio activo que te permita empezar hoy, y dejamos el encargo en marcha por si prefieres volver a tu medicamento habitual en cuanto llegue. La idea es que no te vayas de aquí sin ninguna solución.</t>
         </is>
       </c>
-      <c r="G84" s="14" t="inlineStr">
+      <c r="G84" s="15" t="inlineStr">
         <is>
           <t>Limitarse a decir que lo sientes y que no hay nada que hacer, casi siempre hay alguna vía que explorar antes de rendirse.</t>
         </is>
       </c>
-      <c r="H84" s="14" t="inlineStr">
+      <c r="H84" s="15" t="inlineStr">
         <is>
           <t>Si el tratamiento es para algo agudo, como una infección o dolor importante, priorizar la alternativa inmediata sobre el encargo.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="74" customHeight="1">
-      <c r="A85" s="7" t="n">
+      <c r="A85" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="7" t="inlineStr">
         <is>
           <t>No lo tenemos ahora mismo</t>
         </is>
@@ -4042,62 +4350,62 @@
           <t>Es una opción totalmente razonable, sobre todo si este medicamento lleva tiempo sin regularizarse y no sabemos cuándo va a volver el suministro estable. Si quieres, te puedo comentar qué otras opciones con el mismo efecto existen, para que se lo plantees al médico con la información ya en la mano en vez de ir con la duda de qué pedir. Al final quien tiene que valorar el cambio de tratamiento es el médico, pero yo te puedo ayudar a llegar a esa consulta con las preguntas claras.</t>
         </is>
       </c>
-      <c r="G85" s="10" t="inlineStr">
+      <c r="G85" s="11" t="inlineStr">
         <is>
           <t>Sugerir directamente qué debe recetarle el médico como si fuera decisión tuya, esa parte es del médico.</t>
         </is>
       </c>
-      <c r="H85" s="10" t="inlineStr">
+      <c r="H85" s="11" t="inlineStr">
         <is>
           <t>Ofrecerse a explicar el motivo del desabastecimiento por escrito o de palabra ayuda a que la consulta médica sea más rápida.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="74" customHeight="1">
-      <c r="A86" s="11" t="n">
+      <c r="A86" s="12" t="n">
         <v>82</v>
       </c>
-      <c r="B86" s="12" t="inlineStr">
+      <c r="B86" s="13" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
+      <c r="C86" s="14" t="inlineStr">
         <is>
           <t>«Traigo todas las cajas revueltas, no sé cuál es cuál».</t>
         </is>
       </c>
-      <c r="D86" s="13" t="inlineStr">
+      <c r="D86" s="14" t="inlineStr">
         <is>
           <t>Vamos a mirarlas juntas y le anoto en cada caja cuándo se toma cada una.</t>
         </is>
       </c>
-      <c r="E86" s="13" t="inlineStr">
+      <c r="E86" s="14" t="inlineStr">
         <is>
           <t>Vamos a repasarlas una a una: leo la caja, le pregunto cuándo se la mandó el médico y se la marco con rotulador. Así no depende de acordarse de memoria.</t>
         </is>
       </c>
-      <c r="F86" s="13" t="inlineStr">
+      <c r="F86" s="14" t="inlineStr">
         <is>
           <t>Siéntese un momento, que esto se hace mejor con calma. Vamos sacando las cajas y las separamos por cuándo toca cada una: desayuno, comida, cena. Le apunto en cada caja el horario con rotulador grande, y si quiere le preparo también un pastillero semanal. Así en casa solo tiene que mirar la caja, no memorizar nada.</t>
         </is>
       </c>
-      <c r="G86" s="14" t="inlineStr">
+      <c r="G86" s="15" t="inlineStr">
         <is>
           <t>No le des toda la explicación de golpe y de pie, en ese momento necesita que alguien se siente con ella, no un discurso rápido.</t>
         </is>
       </c>
-      <c r="H86" s="14" t="inlineStr">
+      <c r="H86" s="15" t="inlineStr">
         <is>
           <t>Si además hay más de un médico recetando (cardiólogo, médico de cabecera), avisa al farmacéutico para revisar posibles duplicidades o interacciones.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="74" customHeight="1">
-      <c r="A87" s="7" t="n">
+      <c r="A87" s="8" t="n">
         <v>83</v>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="7" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
@@ -4122,62 +4430,62 @@
           <t>Es muy habitual, no se preocupe. Lo que mejor funciona es un pastillero con los siete días y con mañana y noche separadas: usted lo llena una vez a la semana y luego solo mira si el hueco está vacío o lleno. Si vive sola y le cuesta llenarlo, algún familiar puede hacerlo el domingo para toda la semana. También hay alarmas sencillas en el móvil, si le resulta más cómodo.</t>
         </is>
       </c>
-      <c r="G87" s="10" t="inlineStr">
+      <c r="G87" s="11" t="inlineStr">
         <is>
           <t>No le digas simplemente que tiene que estar más atenta, el problema no es de atención, es de sistema.</t>
         </is>
       </c>
-      <c r="H87" s="10" t="inlineStr">
+      <c r="H87" s="11" t="inlineStr">
         <is>
           <t>Si toma anticoagulante o insulina, el pastillero es aún más importante: una duda de si ya se la tomó hay que resolverla llamando al médico, no adivinando.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="74" customHeight="1">
-      <c r="A88" s="11" t="n">
+      <c r="A88" s="12" t="n">
         <v>84</v>
       </c>
-      <c r="B88" s="12" t="inlineStr">
+      <c r="B88" s="13" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
       </c>
-      <c r="C88" s="13" t="inlineStr">
+      <c r="C88" s="14" t="inlineStr">
         <is>
           <t>«Mi padre toma seis medicamentos, ¿los puede tomar todos juntos?».</t>
         </is>
       </c>
-      <c r="D88" s="13" t="inlineStr">
+      <c r="D88" s="14" t="inlineStr">
         <is>
           <t>La mayoría sí, pero mejor que el farmacéutico revise la combinación exacta con usted.</t>
         </is>
       </c>
-      <c r="E88" s="13" t="inlineStr">
+      <c r="E88" s="14" t="inlineStr">
         <is>
           <t>Depende de cuáles sean exactamente, así que prefiero que lo mire el farmacéutico con la lista completa delante. Si me la trae, se lo comprobamos ahora mismo.</t>
         </is>
       </c>
-      <c r="F88" s="13" t="inlineStr">
+      <c r="F88" s="14" t="inlineStr">
         <is>
           <t>Es una pregunta que hacemos siempre con calma, porque con seis medicamentos puede haber alguno que convenga separar en el horario o que interactúe con otro. Lo mejor es traer la lista completa, con las dosis, y que el farmacéutico la revise entera de una vez, no medicamento a medicamento. De paso aprovechamos para ver si hay algo que ya no hace falta o que se pueda simplificar.</t>
         </is>
       </c>
-      <c r="G88" s="14" t="inlineStr">
+      <c r="G88" s="15" t="inlineStr">
         <is>
           <t>No contestes que sí, tranquilo, todos juntos, sin haber visto la lista real, aunque parezca que tienes prisa.</t>
         </is>
       </c>
-      <c r="H88" s="14" t="inlineStr">
+      <c r="H88" s="15" t="inlineStr">
         <is>
           <t>Una revisión completa de la medicación de un paciente polimedicado es tarea del farmacéutico, no una respuesta rápida de mostrador.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="74" customHeight="1">
-      <c r="A89" s="7" t="n">
+      <c r="A89" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B89" s="7" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
@@ -4202,62 +4510,62 @@
           <t>Entiendo que dé pena tirarlas, pero un medicamento sobrante de hace meses puede corresponder a un tratamiento que ya cambió, o simplemente haber caducado. Antes de retomarlo por su cuenta, mejor que lo veamos aquí: miramos la caja, la fecha, y si coincide con lo que tiene recetado ahora. Si ya no sirve, la puede traer para el punto SIGRE, así no se queda en casa acumulando cajas.</t>
         </is>
       </c>
-      <c r="G89" s="10" t="inlineStr">
+      <c r="G89" s="11" t="inlineStr">
         <is>
           <t>No le restes importancia con un si es lo mismo da igual, los tratamientos cambian de dosis aunque el nombre se parezca.</t>
         </is>
       </c>
-      <c r="H89" s="10" t="inlineStr">
+      <c r="H89" s="11" t="inlineStr">
         <is>
           <t>Cualquier retoma de medicación antigua sin receta vigente pasa por el farmacéutico, nunca se decide en el mostrador a ojo.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="74" customHeight="1">
-      <c r="A90" s="11" t="n">
+      <c r="A90" s="12" t="n">
         <v>86</v>
       </c>
-      <c r="B90" s="12" t="inlineStr">
+      <c r="B90" s="13" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
       </c>
-      <c r="C90" s="13" t="inlineStr">
+      <c r="C90" s="14" t="inlineStr">
         <is>
           <t>«Desde que tomo la pastilla nueva del médico me noto mareado».</t>
         </is>
       </c>
-      <c r="D90" s="13" t="inlineStr">
+      <c r="D90" s="14" t="inlineStr">
         <is>
           <t>Eso hay que decírselo al médico cuanto antes, no lo deje pasar.</t>
         </is>
       </c>
-      <c r="E90" s="13" t="inlineStr">
+      <c r="E90" s="14" t="inlineStr">
         <is>
           <t>Un mareo que empieza justo con un medicamento nuevo tiene que valorarlo el médico, puede ser el fármaco, la dosis o algo distinto. Llame a su centro de salud y cuénteselo.</t>
         </is>
       </c>
-      <c r="F90" s="13" t="inlineStr">
+      <c r="F90" s="14" t="inlineStr">
         <is>
           <t>Hace usted bien en contarlo, esto no hay que dejarlo pasar. Cuando un síntoma nuevo coincide con el inicio de un medicamento, lo correcto es que lo valore quien se lo ha recetado, porque puede ser la dosis, puede ser el propio fármaco o puede ser otra cosa distinta que conviene descartar. Mientras tanto, no deje de tomarlo por su cuenta sin hablar antes con el médico, salvo que el mareo sea muy fuerte, en cuyo caso vaya a urgencias.</t>
         </is>
       </c>
-      <c r="G90" s="14" t="inlineStr">
+      <c r="G90" s="15" t="inlineStr">
         <is>
           <t>No le digas que es normal y que ya se le pasará, un síntoma nuevo con un fármaco nuevo se deriva, no se minimiza.</t>
         </is>
       </c>
-      <c r="H90" s="14" t="inlineStr">
+      <c r="H90" s="15" t="inlineStr">
         <is>
           <t>Mareo con caídas, confusión o pérdida de fuerza es señal de alarma: en ese caso no se espera a la próxima cita, se deriva de forma urgente.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="74" customHeight="1">
-      <c r="A91" s="7" t="n">
+      <c r="A91" s="8" t="n">
         <v>87</v>
       </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="B91" s="7" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
@@ -4282,62 +4590,62 @@
           <t>Es una pregunta muy razonable, pero la respuesta depende del medicamento exacto. Hay pastillas con una ranura pensada para partirse y otras con una cubierta especial que, si se rompe, hace que se libere de golpe o se estropee. Déjeme comprobarlo con la caja delante. Si esta no se puede partir, hay alternativas: formato en gotas, en sobres, o hablar con el médico para cambiar la presentación.</t>
         </is>
       </c>
-      <c r="G91" s="10" t="inlineStr">
+      <c r="G91" s="11" t="inlineStr">
         <is>
           <t>No asumas que si es pequeña se puede partir, el tamaño no dice nada sobre si tiene cubierta especial.</t>
         </is>
       </c>
-      <c r="H91" s="10" t="inlineStr">
+      <c r="H91" s="11" t="inlineStr">
         <is>
           <t>Si la dificultad para tragar es reciente o va a más, coméntaselo también al médico, puede ser algo a revisar aparte de la solución práctica.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="74" customHeight="1">
-      <c r="A92" s="11" t="n">
+      <c r="A92" s="12" t="n">
         <v>88</v>
       </c>
-      <c r="B92" s="12" t="inlineStr">
+      <c r="B92" s="13" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
+      <c r="C92" s="14" t="inlineStr">
         <is>
           <t>«Soy la cuidadora, ¿cómo organizo esto para toda la semana?».</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="D92" s="14" t="inlineStr">
         <is>
           <t>Con un pastillero de siete días y mañana, tarde y noche lo tiene resuelto de un vistazo.</t>
         </is>
       </c>
-      <c r="E92" s="13" t="inlineStr">
+      <c r="E92" s="14" t="inlineStr">
         <is>
           <t>Un pastillero semanal con los tres momentos del día separados es lo más práctico. Lo rellena una vez y luego solo comprueba que cada hueco esté vacío cuando toca.</t>
         </is>
       </c>
-      <c r="F92" s="13" t="inlineStr">
+      <c r="F92" s="14" t="inlineStr">
         <is>
           <t>Lo mejor para un cuidador es quitarse la carga de la memoria y ponerla en un sistema visual. Un pastillero de siete días, con mañana, tarde y noche, se rellena una vez por semana con calma, comprobando cada caja contra la pauta del médico. Si la persona toma medicación variable, conviene apuntar también la pauta en un papel al lado del pastillero. Y si hay algún cambio de tratamiento, mejor rehacer el pastillero entero esa semana.</t>
         </is>
       </c>
-      <c r="G92" s="14" t="inlineStr">
+      <c r="G92" s="15" t="inlineStr">
         <is>
           <t>No des por hecho que el cuidador conoce la pauta de memoria, mejor confirmar cada medicamento con la caja en la mano.</t>
         </is>
       </c>
-      <c r="H92" s="14" t="inlineStr">
+      <c r="H92" s="15" t="inlineStr">
         <is>
           <t>Si hay varios cuidadores turnándose, un cuaderno o nota compartida de quién ha dado qué evita duplicar o saltarse tomas.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="74" customHeight="1">
-      <c r="A93" s="7" t="n">
+      <c r="A93" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
@@ -4362,62 +4670,62 @@
           <t>Le agradezco que lo pregunte antes de comprarlo, porque es justo el tipo de combinación que hay que evitar: los antiinflamatorios interfieren con el anticoagulante y suben el riesgo de sangrado, incluso en formato tópico hay que tener cuidado. Para el dolor de rodilla hay alternativas que no interaccionan igual, y el farmacéutico le puede orientar según lo que le venga mejor. Si el dolor es intenso o viene de un golpe, coméntelo también con su médico.</t>
         </is>
       </c>
-      <c r="G93" s="10" t="inlineStr">
+      <c r="G93" s="11" t="inlineStr">
         <is>
           <t>No despaches esto con un tome lo que quiera, es de venta libre, la venta libre no significa que sea compatible con todo.</t>
         </is>
       </c>
-      <c r="H93" s="10" t="inlineStr">
+      <c r="H93" s="11" t="inlineStr">
         <is>
           <t>Cualquier paciente con Sintrom o similares es bandera roja automática para antiinflamatorios: pasa siempre por el farmacéutico antes de vender.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="74" customHeight="1">
-      <c r="A94" s="11" t="n">
+      <c r="A94" s="12" t="n">
         <v>90</v>
       </c>
-      <c r="B94" s="12" t="inlineStr">
+      <c r="B94" s="13" t="inlineStr">
         <is>
           <t>Mayores y polimedicación</t>
         </is>
       </c>
-      <c r="C94" s="13" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
         <is>
           <t>«No me acuerdo si ya me he tomado la de la tensión de hoy».</t>
         </is>
       </c>
-      <c r="D94" s="13" t="inlineStr">
+      <c r="D94" s="14" t="inlineStr">
         <is>
           <t>Si tiene dudas, mejor no repetir dosis, consulte antes de tomar otra.</t>
         </is>
       </c>
-      <c r="E94" s="13" t="inlineStr">
+      <c r="E94" s="14" t="inlineStr">
         <is>
           <t>Ante la duda, no conviene tomar una segunda dosis por si acaso. Mejor esperar a la próxima toma y, si repite esta situación, ponemos un sistema para no perder la cuenta.</t>
         </is>
       </c>
-      <c r="F94" s="13" t="inlineStr">
+      <c r="F94" s="14" t="inlineStr">
         <is>
           <t>Es mejor no arriesgarse a duplicar la dosis, sobre todo con medicación para la tensión. Si de verdad no lo sabe, lo prudente es dejarlo para la siguiente toma programada y vigilar cómo se encuentra durante el día. Para que esto no se repita, le recomiendo un pastillero semanal o marcar la caja según se va tomando cada pastilla, así lo ve a simple vista sin depender de la memoria.</t>
         </is>
       </c>
-      <c r="G94" s="14" t="inlineStr">
+      <c r="G94" s="15" t="inlineStr">
         <is>
           <t>No le digas que se la tome otra vez, mejor pasarse que quedarse corto, con antihipertensivos una dosis doble sí importa.</t>
         </is>
       </c>
-      <c r="H94" s="14" t="inlineStr">
+      <c r="H94" s="15" t="inlineStr">
         <is>
           <t>Si nota mareo o el corazón muy acelerado después de una posible duplicidad, debe consultar sin esperar.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="74" customHeight="1">
-      <c r="A95" s="7" t="n">
+      <c r="A95" s="8" t="n">
         <v>91</v>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
@@ -4442,62 +4750,62 @@
           <t>Entiendo que quieras solucionarlo ya, pero cinco días de fiebre junto con tos es más de lo que se espera de un catarro normal, y conviene descartar que sea otra cosa que necesite tratamiento distinto. Te recomiendo pedir cita con tu médico o, si la fiebre sube mucho o te cuesta respirar, ir directamente a urgencias. Mientras tanto te puedo recomendar algo para la tos y para bajar la fiebre, pero como alivio, no como solución.</t>
         </is>
       </c>
-      <c r="G95" s="10" t="inlineStr">
+      <c r="G95" s="11" t="inlineStr">
         <is>
           <t>No vendas nada pensado para que se te quite ya sin más, eso no lo decides tú en el mostrador y sin diagnóstico es un riesgo.</t>
         </is>
       </c>
-      <c r="H95" s="10" t="inlineStr">
+      <c r="H95" s="11" t="inlineStr">
         <is>
           <t>Fiebre alta que no baja con antitérmico, o dificultad para respirar, es motivo de urgencias, no de cita programada.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="74" customHeight="1">
-      <c r="A96" s="11" t="n">
+      <c r="A96" s="12" t="n">
         <v>92</v>
       </c>
-      <c r="B96" s="12" t="inlineStr">
+      <c r="B96" s="13" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
       </c>
-      <c r="C96" s="13" t="inlineStr">
+      <c r="C96" s="14" t="inlineStr">
         <is>
           <t>«Me ha dado un dolor de cabeza muy fuerte de golpe, no es como el que tengo normalmente».</t>
         </is>
       </c>
-      <c r="D96" s="13" t="inlineStr">
+      <c r="D96" s="14" t="inlineStr">
         <is>
           <t>Ese dolor tan distinto al habitual hay que consultarlo ya, no esperes.</t>
         </is>
       </c>
-      <c r="E96" s="13" t="inlineStr">
+      <c r="E96" s="14" t="inlineStr">
         <is>
           <t>Un dolor de cabeza brusco y mucho más fuerte de lo normal no es para esperar a ver si se pasa. Te recomiendo ir a urgencias o llamar al médico ahora mismo.</t>
         </is>
       </c>
-      <c r="F96" s="13" t="inlineStr">
+      <c r="F96" s="14" t="inlineStr">
         <is>
           <t>Cuando el dolor de cabeza aparece de golpe y es claramente distinto al que sueles tener, es una señal que hay que tomarse en serio, no algo para calmar con un analgésico y seguir el día. Lo prudente es que lo valoren cuanto antes, en tu centro de salud si te dan cita hoy, o en urgencias si no. No te voy a dar nada para el dolor sin que antes lo hayan visto, porque enmascararía lo que está pasando.</t>
         </is>
       </c>
-      <c r="G96" s="14" t="inlineStr">
+      <c r="G96" s="15" t="inlineStr">
         <is>
           <t>No le des un analgésico fuerte para que aguante sin decirle que consulte, eso retrasa la valoración.</t>
         </is>
       </c>
-      <c r="H96" s="14" t="inlineStr">
+      <c r="H96" s="15" t="inlineStr">
         <is>
           <t>Si además hay visión borrosa, dificultad para hablar o pérdida de fuerza en un lado, es urgencia inmediata, se llama al 112.</t>
         </is>
       </c>
     </row>
     <row r="97" ht="74" customHeight="1">
-      <c r="A97" s="7" t="n">
+      <c r="A97" s="8" t="n">
         <v>93</v>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
@@ -4522,62 +4830,62 @@
           <t>Este es uno de los síntomas que no se trata en la farmacia bajo ningún concepto, porque puede tener muchas causas y algunas son graves. Lo que te pido es que vayas a urgencias ahora, no esperes a ver si se pasa solo. Si el dolor va a más, se extiende al brazo o la mandíbula, o te falta el aire, llama directamente al 112 en vez de ir por tu cuenta.</t>
         </is>
       </c>
-      <c r="G97" s="10" t="inlineStr">
+      <c r="G97" s="11" t="inlineStr">
         <is>
           <t>No preguntes demasiado ni intentes filtrar tú si es grave o no, cualquier dolor torácico se deriva sin dilación.</t>
         </is>
       </c>
-      <c r="H97" s="10" t="inlineStr">
+      <c r="H97" s="11" t="inlineStr">
         <is>
           <t>Este es de los pocos casos donde no se pierde tiempo explicando alternativas, se deriva de inmediato y se acompaña si hace falta.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="74" customHeight="1">
-      <c r="A98" s="11" t="n">
+      <c r="A98" s="12" t="n">
         <v>94</v>
       </c>
-      <c r="B98" s="12" t="inlineStr">
+      <c r="B98" s="13" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
       </c>
-      <c r="C98" s="13" t="inlineStr">
+      <c r="C98" s="14" t="inlineStr">
         <is>
           <t>«Tengo esta herida en la pierna desde hace semanas y no acaba de cerrar».</t>
         </is>
       </c>
-      <c r="D98" s="13" t="inlineStr">
+      <c r="D98" s="14" t="inlineStr">
         <is>
           <t>Una herida que no cicatriza en semanas la tiene que ver el médico.</t>
         </is>
       </c>
-      <c r="E98" s="13" t="inlineStr">
+      <c r="E98" s="14" t="inlineStr">
         <is>
           <t>Si lleva tanto tiempo sin cerrar, conviene que la vea el médico o el enfermero de tu centro de salud, puede necesitar otro tratamiento. Te ayudo a limpiarla mientras tanto.</t>
         </is>
       </c>
-      <c r="F98" s="13" t="inlineStr">
+      <c r="F98" s="14" t="inlineStr">
         <is>
           <t>Una herida que no evoluciona en varias semanas ya no es algo que se resuelva solo con la crema adecuada, hay que ver por qué no cierra, y eso pasa por que la valore un profesional sanitario que pueda explorarla. Puede ser algo circulatorio, algo relacionado con otra condición de salud, o simplemente necesitar una cura distinta. Te doy algo para mantenerla limpia hoy, pero pide cita con enfermería o con tu médico esta semana.</t>
         </is>
       </c>
-      <c r="G98" s="14" t="inlineStr">
+      <c r="G98" s="15" t="inlineStr">
         <is>
           <t>No sigas recomendando cremas distintas semana tras semana sin decir nada, ese patrón es justo la señal de que hace falta derivar.</t>
         </is>
       </c>
-      <c r="H98" s="14" t="inlineStr">
+      <c r="H98" s="15" t="inlineStr">
         <is>
           <t>Si la herida está caliente, muy enrojecida alrededor, con mal olor o supura, la derivación es prioritaria, no puede esperar a la semana que viene.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="74" customHeight="1">
-      <c r="A99" s="7" t="n">
+      <c r="A99" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
@@ -4602,62 +4910,62 @@
           <t>En niños pequeños la fiebre alta que se mantiene toda la noche es motivo para que lo vea el pediatra, no solo para manejarla en casa. Te explico bien la dosis del antitérmico según su peso mientras organizáis la visita, pero eso es un alivio puntual, no sustituye la valoración. Si además está muy decaído, le cuesta respirar, tiene manchas en la piel o no hay manera de bajarle la fiebre, id a urgencias directamente.</t>
         </is>
       </c>
-      <c r="G99" s="10" t="inlineStr">
+      <c r="G99" s="11" t="inlineStr">
         <is>
           <t>No minimices diciendo que los niños cogen fiebre por todo, en menores de tres meses o fiebre muy alta y mantenida no se resta importancia.</t>
         </is>
       </c>
-      <c r="H99" s="10" t="inlineStr">
+      <c r="H99" s="11" t="inlineStr">
         <is>
           <t>Fiebre en un bebé de menos de tres meses es siempre derivación urgente, sin excepción, aunque parezca que está bien.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="74" customHeight="1">
-      <c r="A100" s="11" t="n">
+      <c r="A100" s="12" t="n">
         <v>96</v>
       </c>
-      <c r="B100" s="12" t="inlineStr">
+      <c r="B100" s="13" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
+      <c r="C100" s="14" t="inlineStr">
         <is>
           <t>«Llevo cuatro días con diarrea y ya no sé qué tomar».</t>
         </is>
       </c>
-      <c r="D100" s="13" t="inlineStr">
+      <c r="D100" s="14" t="inlineStr">
         <is>
           <t>Cuatro días es demasiado, mejor que te vea el médico antes de seguir probando cosas.</t>
         </is>
       </c>
-      <c r="E100" s="13" t="inlineStr">
+      <c r="E100" s="14" t="inlineStr">
         <is>
           <t>A partir de unos días de diarrea seguida conviene descartar que sea algo que necesite tratamiento específico, sobre todo si notas signos de deshidratación. Te recomiendo consultar y cuidar líquidos y sales.</t>
         </is>
       </c>
-      <c r="F100" s="13" t="inlineStr">
+      <c r="F100" s="14" t="inlineStr">
         <is>
           <t>Cuatro días de diarrea ya no entra dentro de lo que se resuelve solo con dieta y algún producto de farmacia, hay que ver qué lo está causando, sobre todo si notas boca seca, mareo al levantarte o orinas muy poco, señales de deshidratación. Te recomiendo pedir cita con tu médico esta semana, y si aparece sangre en las heces, fiebre alta o el mareo es fuerte, mejor ir a urgencias directamente. Mientras tanto, sueros de rehidratación y evitar lácteos y grasas te pueden ayudar.</t>
         </is>
       </c>
-      <c r="G100" s="14" t="inlineStr">
+      <c r="G100" s="15" t="inlineStr">
         <is>
           <t>No sigas cambiando de producto probiótico o antidiarreico sin límite, si no mejora en unos días el problema es de derivación, no de elegir mejor marca.</t>
         </is>
       </c>
-      <c r="H100" s="14" t="inlineStr">
+      <c r="H100" s="15" t="inlineStr">
         <is>
           <t>En niños pequeños y personas mayores, la deshidratación avanza mucho más rápido: el margen para derivar es más corto que en un adulto sano.</t>
         </is>
       </c>
     </row>
     <row r="101" ht="74" customHeight="1">
-      <c r="A101" s="7" t="n">
+      <c r="A101" s="8" t="n">
         <v>97</v>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="7" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
@@ -4682,62 +4990,62 @@
           <t>Una erupción que avanza en cuestión de horas o días es distinta de una irritación puntual, y conviene que la vea el médico para identificar la causa, porque el tratamiento cambia mucho según de qué se trate. Te puedo recomendar algo para calmar el picor mientras consigues cita, pero no te doy nada que pueda enmascarar cómo evoluciona la piel de cara al diagnóstico. Si además notas hinchazón en la cara o los labios, o te cuesta respirar, eso es urgencia inmediata.</t>
         </is>
       </c>
-      <c r="G101" s="10" t="inlineStr">
+      <c r="G101" s="11" t="inlineStr">
         <is>
           <t>No des una crema con corticoide sin más explicación cuando la lesión está cambiando rápido, puede tapar signos que el médico necesita ver.</t>
         </is>
       </c>
-      <c r="H101" s="10" t="inlineStr">
+      <c r="H101" s="11" t="inlineStr">
         <is>
           <t>Hinchazón de cara, labios o garganta junto con la erupción es señal de alarma y se deriva a urgencias, no a la consulta programada.</t>
         </is>
       </c>
     </row>
     <row r="102" ht="74" customHeight="1">
-      <c r="A102" s="11" t="n">
+      <c r="A102" s="12" t="n">
         <v>98</v>
       </c>
-      <c r="B102" s="12" t="inlineStr">
+      <c r="B102" s="13" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
       </c>
-      <c r="C102" s="13" t="inlineStr">
+      <c r="C102" s="14" t="inlineStr">
         <is>
           <t>«Tengo un dolor fuerte aquí en el costado, como un pinchazo, no se me pasa».</t>
         </is>
       </c>
-      <c r="D102" s="13" t="inlineStr">
+      <c r="D102" s="14" t="inlineStr">
         <is>
           <t>Ese dolor localizado y fuerte hay que descartarlo en el médico, no lo aguantes en casa.</t>
         </is>
       </c>
-      <c r="E102" s="13" t="inlineStr">
+      <c r="E102" s="14" t="inlineStr">
         <is>
           <t>Un dolor así, fuerte y en un punto concreto, conviene que lo valoren, puede tener varios orígenes y algunos necesitan atención pronto. Mejor consulta hoy, o urgencias si va a más.</t>
         </is>
       </c>
-      <c r="F102" s="13" t="inlineStr">
+      <c r="F102" s="14" t="inlineStr">
         <is>
           <t>Cuando el dolor es intenso, está bien localizado y no cede, es preferible que lo valore un médico antes que intentar aliviarlo por tu cuenta, porque puede tratarse de algo que necesite pruebas para saber qué es exactamente. Si el dolor es tan fuerte que no te deja hacer vida normal, si viene con fiebre, con vómitos, o si notas que va a más, no esperes a mañana, ve a urgencias. Te puedo dar algo suave mientras te desplazas, pero la prioridad es que te vean.</t>
         </is>
       </c>
-      <c r="G102" s="14" t="inlineStr">
+      <c r="G102" s="15" t="inlineStr">
         <is>
           <t>No le restes gravedad diciendo que seguro que es una contractura, sin explorar no se puede saber y el riesgo de equivocarse es alto.</t>
         </is>
       </c>
-      <c r="H102" s="14" t="inlineStr">
+      <c r="H102" s="15" t="inlineStr">
         <is>
           <t>Dolor abdominal muy intenso, rígido al tacto o con vómitos persistentes es siempre derivación urgente.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="74" customHeight="1">
-      <c r="A103" s="7" t="n">
+      <c r="A103" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B103" s="7" t="inlineStr">
         <is>
           <t>Cuando hay que derivar al médico</t>
         </is>
@@ -4762,62 +5070,62 @@
           <t>Esto es una urgencia real y el tiempo importa: la hinchazón en la cara tras comer algo puede evolucionar rápido y afectar a la respiración, así que no es momento de buscar un antihistamínico en el mostrador. Llama al 112 o ve a urgencias inmediatamente, y si notas que te cuesta tragar o respirar, dilo nada más llegar. No pierdas tiempo esperando a ver si mejora sola.</t>
         </is>
       </c>
-      <c r="G103" s="10" t="inlineStr">
+      <c r="G103" s="11" t="inlineStr">
         <is>
           <t>No entretengas al paciente buscando un antihistamínico en la estantería, en una reacción que avanza cada minuto cuenta.</t>
         </is>
       </c>
-      <c r="H103" s="10" t="inlineStr">
+      <c r="H103" s="11" t="inlineStr">
         <is>
           <t>Cualquier signo de hinchazón facial, de labios o de garganta tras comer o tomar un medicamento es derivación urgente inmediata, sin pasos intermedios.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="74" customHeight="1">
-      <c r="A104" s="11" t="n">
+      <c r="A104" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="B104" s="12" t="inlineStr">
+      <c r="B104" s="13" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
       </c>
-      <c r="C104" s="13" t="inlineStr">
+      <c r="C104" s="14" t="inlineStr">
         <is>
           <t>«Llevo veinte minutos esperando, ¿esto es normal?».</t>
         </is>
       </c>
-      <c r="D104" s="13" t="inlineStr">
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>Tienes razón, hoy está siendo mucho, ya te atiendo yo.</t>
         </is>
       </c>
-      <c r="E104" s="13" t="inlineStr">
+      <c r="E104" s="14" t="inlineStr">
         <is>
           <t>Tienes razón, la espera de hoy se ha alargado más de la cuenta. Ya te atiendo yo, dime qué necesitas y lo resolvemos ahora mismo.</t>
         </is>
       </c>
-      <c r="F104" s="13" t="inlineStr">
+      <c r="F104" s="14" t="inlineStr">
         <is>
           <t>Entiendo que veinte minutos es mucho tiempo de pie esperando, y tienes razón en decirlo. Hoy se han acumulado varias cosas seguidas, pero eso no quita que la espera sea larga. Vamos, dime qué necesitas, que te atiendo yo ya y lo resolvemos rápido. Si quieres dejar el pedido y volver luego a recogerlo, también podemos hacerlo así.</t>
         </is>
       </c>
-      <c r="G104" s="14" t="inlineStr">
+      <c r="G104" s="15" t="inlineStr">
         <is>
           <t>No digas es que hay mucha gente como si fuera excusa suficiente, reconoce la espera antes de explicar el motivo.</t>
         </is>
       </c>
-      <c r="H104" s="14" t="inlineStr">
+      <c r="H104" s="15" t="inlineStr">
         <is>
           <t>Si la espera larga se repite a las mismas horas, coméntalo al titular: es un problema de turnos o de personal, no algo que se arregle disculpándose cada día.</t>
         </is>
       </c>
     </row>
     <row r="105" ht="74" customHeight="1">
-      <c r="A105" s="7" t="n">
+      <c r="A105" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="B105" s="8" t="inlineStr">
+      <c r="B105" s="7" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
@@ -4842,62 +5150,62 @@
           <t>Entiendo que el precio te sorprenda, y no es una cifra que decidamos aquí: depende de la aportación que te corresponde según el tipo de receta y del propio precio del medicamento. Si quieres, te explico por qué esta caja concreta cuesta esto, y si hay una alternativa con la misma composición y otro precio, te la comento también. A veces cambiar de formato o de presentación reduce el gasto sin cambiar el tratamiento.</t>
         </is>
       </c>
-      <c r="G105" s="10" t="inlineStr">
+      <c r="G105" s="11" t="inlineStr">
         <is>
           <t>No respondas eso lo pone Sanidad, yo no puedo hacer nada, como si zanjaras la conversación, explica y busca alternativas si las hay.</t>
         </is>
       </c>
-      <c r="H105" s="10" t="inlineStr">
+      <c r="H105" s="11" t="inlineStr">
         <is>
           <t>Si hay una alternativa más económica con el mismo principio activo, ofrécela siempre antes de que el paciente se vaya con la sensación de que no había opción.</t>
         </is>
       </c>
     </row>
     <row r="106" ht="74" customHeight="1">
-      <c r="A106" s="11" t="n">
+      <c r="A106" s="12" t="n">
         <v>102</v>
       </c>
-      <c r="B106" s="12" t="inlineStr">
+      <c r="B106" s="13" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
       </c>
-      <c r="C106" s="13" t="inlineStr">
+      <c r="C106" s="14" t="inlineStr">
         <is>
           <t>«Esto que me diste la otra vez no me ha hecho nada».</t>
         </is>
       </c>
-      <c r="D106" s="13" t="inlineStr">
+      <c r="D106" s="14" t="inlineStr">
         <is>
           <t>Vaya, cuéntame qué notaste y vemos si conviene probar otra cosa.</t>
         </is>
       </c>
-      <c r="E106" s="13" t="inlineStr">
+      <c r="E106" s="14" t="inlineStr">
         <is>
           <t>Lamento que no te haya ido bien. Cuéntame exactamente qué síntomas tenías y cuánto tiempo lo usaste, así vemos si conviene otro producto o si lo mira el médico.</t>
         </is>
       </c>
-      <c r="F106" s="13" t="inlineStr">
+      <c r="F106" s="14" t="inlineStr">
         <is>
           <t>Vaya, siento que no te haya funcionado como esperabas. Antes de recomendarte otra cosa, cuéntame bien qué te pasaba, durante cuánto tiempo usaste el producto y cómo lo usaste, porque a veces el resultado depende de la constancia o de la forma de aplicarlo. Con esa información vemos si tiene sentido probar una alternativa distinta, o si lo que tienes conviene que lo valore el médico porque no es lo que parecía en un principio.</t>
         </is>
       </c>
-      <c r="G106" s="14" t="inlineStr">
+      <c r="G106" s="15" t="inlineStr">
         <is>
           <t>No te pongas a la defensiva con un a todo el mundo le funciona, la experiencia del paciente es el punto de partida, no algo que rebatir.</t>
         </is>
       </c>
-      <c r="H106" s="14" t="inlineStr">
+      <c r="H106" s="15" t="inlineStr">
         <is>
           <t>Si el síntoma inicial no ha mejorado nada en el plazo esperable, es más señal de derivar que de cambiar de producto sin más.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="74" customHeight="1">
-      <c r="A107" s="7" t="n">
+      <c r="A107" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="B107" s="8" t="inlineStr">
+      <c r="B107" s="7" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
@@ -4922,62 +5230,62 @@
           <t>Gracias por decírmelo enseguida, esto hay que arreglarlo ya. Déjame ver la caja que tienes y la que te correspondía, para entender dónde se ha cruzado. Te doy la correcta ahora mismo y no te cobro de más por el cambio. Si has llegado a tomarte algo de la caja equivocada, dímelo también, porque eso lo consultamos con el farmacéutico para asegurarnos.</t>
         </is>
       </c>
-      <c r="G107" s="10" t="inlineStr">
+      <c r="G107" s="11" t="inlineStr">
         <is>
           <t>No minimices con un bueno, tampoco es tan grave, un error de dispensación se reconoce y se corrige sin restarle importancia.</t>
         </is>
       </c>
-      <c r="H107" s="10" t="inlineStr">
+      <c r="H107" s="11" t="inlineStr">
         <is>
           <t>Si el paciente ha tomado ya alguna dosis del producto equivocado, es el farmacéutico quien valora si hay que hacer algo más, no se cierra el tema con la disculpa.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="74" customHeight="1">
-      <c r="A108" s="11" t="n">
+      <c r="A108" s="12" t="n">
         <v>104</v>
       </c>
-      <c r="B108" s="12" t="inlineStr">
+      <c r="B108" s="13" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
       </c>
-      <c r="C108" s="13" t="inlineStr">
+      <c r="C108" s="14" t="inlineStr">
         <is>
           <t>«Tu compañera me atendió fatal el otro día, muy borde».</t>
         </is>
       </c>
-      <c r="D108" s="13" t="inlineStr">
+      <c r="D108" s="14" t="inlineStr">
         <is>
           <t>Siento que te sintieras así, lo traslado y lo hablamos internamente.</t>
         </is>
       </c>
-      <c r="E108" s="13" t="inlineStr">
+      <c r="E108" s="14" t="inlineStr">
         <is>
           <t>Siento que te haya pasado eso, no es lo que buscamos. Lo comento con el equipo para que no se repita, y hoy me encargo yo de que salgas contento.</t>
         </is>
       </c>
-      <c r="F108" s="13" t="inlineStr">
+      <c r="F108" s="14" t="inlineStr">
         <is>
           <t>Siento mucho que tuvieras esa sensación, no es lo que queremos que se lleve nadie de aquí. Voy a comentarlo con el equipo, porque nos interesa saber cuándo algo no ha ido bien para poder corregirlo. Hoy me ocupo yo de que la visita vaya como debe ser, dime qué necesitas. Y si en algún momento quieres hablarlo también con el titular, encantados de escucharte.</t>
         </is>
       </c>
-      <c r="G108" s="14" t="inlineStr">
+      <c r="G108" s="15" t="inlineStr">
         <is>
           <t>No defiendas ni critiques a la compañera delante del cliente, ese tema se gestiona luego, dentro del equipo.</t>
         </is>
       </c>
-      <c r="H108" s="14" t="inlineStr">
+      <c r="H108" s="15" t="inlineStr">
         <is>
           <t>Estas quejas se anotan y se comentan en privado con la persona implicada, nunca se resuelven ni se juzgan en el mostrador delante de otros clientes.</t>
         </is>
       </c>
     </row>
     <row r="109" ht="74" customHeight="1">
-      <c r="A109" s="7" t="n">
+      <c r="A109" s="8" t="n">
         <v>105</v>
       </c>
-      <c r="B109" s="8" t="inlineStr">
+      <c r="B109" s="7" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
@@ -5002,62 +5310,62 @@
           <t>Veo que estás muy molesto, y quiero entender bien qué ha pasado para poder ayudarte. Vamos a hablarlo con calma, aquí me tienes escuchando. Cuéntame desde el principio qué ha ocurrido, sin prisa, y en cuanto lo tenga claro te digo qué podemos hacer. Si prefieres que lo hablemos aparte del mostrador, con más tranquilidad, también podemos pasar a un lado.</t>
         </is>
       </c>
-      <c r="G109" s="10" t="inlineStr">
+      <c r="G109" s="11" t="inlineStr">
         <is>
           <t>No subas tú también el tono ni respondas con un no hace falta gritar, eso suele escalar la situación en vez de bajarla.</t>
         </is>
       </c>
-      <c r="H109" s="10" t="inlineStr">
+      <c r="H109" s="11" t="inlineStr">
         <is>
           <t>Si el cliente no baja el tono y hay otros clientes delante, invita a pasar a una zona más apartada; si la situación se descontrola, es el titular quien debe intervenir.</t>
         </is>
       </c>
     </row>
     <row r="110" ht="74" customHeight="1">
-      <c r="A110" s="11" t="n">
+      <c r="A110" s="12" t="n">
         <v>106</v>
       </c>
-      <c r="B110" s="12" t="inlineStr">
+      <c r="B110" s="13" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
       </c>
-      <c r="C110" s="13" t="inlineStr">
+      <c r="C110" s="14" t="inlineStr">
         <is>
           <t>«No quiero el genérico, dame la marca de siempre».</t>
         </is>
       </c>
-      <c r="D110" s="13" t="inlineStr">
+      <c r="D110" s="14" t="inlineStr">
         <is>
           <t>Claro, si la marca está disponible te la doy sin problema.</t>
         </is>
       </c>
-      <c r="E110" s="13" t="inlineStr">
+      <c r="E110" s="14" t="inlineStr">
         <is>
           <t>Sin problema, si tienes preferencia por la marca te la doy, solo dime si hay diferencia de precio y te lo explico antes de cobrarte.</t>
         </is>
       </c>
-      <c r="F110" s="13" t="inlineStr">
+      <c r="F110" s="14" t="inlineStr">
         <is>
           <t>Por supuesto, entiendo que quieras seguir con lo que ya conoces. La composición del genérico es la misma, pero si prefieres la marca de siempre no hay ningún problema en dártela, siempre que esté disponible. Eso sí, puede que haya una diferencia de precio entre una y otra, te lo digo antes de cobrarte para que no haya sorpresa. Si alguna vez notaras que un cambio de marca te sienta distinto, coméntaselo al farmacéutico.</t>
         </is>
       </c>
-      <c r="G110" s="14" t="inlineStr">
+      <c r="G110" s="15" t="inlineStr">
         <is>
           <t>No insistas en el genérico como si el paciente estuviera equivocado, la decisión final sobre marca es suya cuando hay opción.</t>
         </is>
       </c>
-      <c r="H110" s="14" t="inlineStr">
+      <c r="H110" s="15" t="inlineStr">
         <is>
           <t>Si hay sustitución obligada por normativa o falta de stock de la marca, explícalo como un hecho, no como una opinión tuya.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="74" customHeight="1">
-      <c r="A111" s="7" t="n">
+      <c r="A111" s="8" t="n">
         <v>107</v>
       </c>
-      <c r="B111" s="8" t="inlineStr">
+      <c r="B111" s="7" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
@@ -5082,52 +5390,52 @@
           <t>Tiene sentido que lo preguntes si ves una diferencia, vamos a revisarlo bien. Enséñame el ticket de hoy y, si tienes el anterior, lo comparamos línea por línea para ver qué ha variado, puede ser un cambio de precio, de aportación, o efectivamente un error nuestro. Si es un error, lo corregimos y te devolvemos la diferencia que corresponda. Si el cambio viene de fuera, te lo explico para que quede claro.</t>
         </is>
       </c>
-      <c r="G111" s="10" t="inlineStr">
+      <c r="G111" s="11" t="inlineStr">
         <is>
           <t>No respondas el sistema no falla sin comprobar nada, comprueba primero y luego explica.</t>
         </is>
       </c>
-      <c r="H111" s="10" t="inlineStr">
+      <c r="H111" s="11" t="inlineStr">
         <is>
           <t>Si el error se repite con el mismo producto varias veces, avisa al titular para revisar si hay un fallo en el sistema de facturación, no solo el caso puntual.</t>
         </is>
       </c>
     </row>
     <row r="112" ht="74" customHeight="1">
-      <c r="A112" s="11" t="n">
+      <c r="A112" s="12" t="n">
         <v>108</v>
       </c>
-      <c r="B112" s="12" t="inlineStr">
+      <c r="B112" s="13" t="inlineStr">
         <is>
           <t>Quejas y momentos incómodos</t>
         </is>
       </c>
-      <c r="C112" s="13" t="inlineStr">
+      <c r="C112" s="14" t="inlineStr">
         <is>
           <t>«Necesito esto ya y me decís que no hay, ¿cómo puede ser?».</t>
         </is>
       </c>
-      <c r="D112" s="13" t="inlineStr">
+      <c r="D112" s="14" t="inlineStr">
         <is>
           <t>Lo siento, hoy no tenemos, pero te digo dónde lo puedes encontrar ahora mismo.</t>
         </is>
       </c>
-      <c r="E112" s="13" t="inlineStr">
+      <c r="E112" s="14" t="inlineStr">
         <is>
           <t>Siento que justo hoy no tengamos, entiendo que lo necesites ya. Miro si alguna farmacia cercana lo tiene en stock y, si quieres, te lo pedimos para mañana.</t>
         </is>
       </c>
-      <c r="F112" s="13" t="inlineStr">
+      <c r="F112" s="14" t="inlineStr">
         <is>
           <t>Entiendo la urgencia, y siento que justo hoy no lo tengamos en el mostrador. Voy a mirar si alguna farmacia cercana lo tiene disponible ahora mismo para que no pierdas tiempo. Si no lo encontramos así, te lo pedimos con carácter urgente y en cuanto llegue te avisamos, normalmente para mañana a primera hora. Si es algo que no puede esperar en absoluto, dime el motivo y vemos entre las opciones cuál es la más rápida.</t>
         </is>
       </c>
-      <c r="G112" s="14" t="inlineStr">
+      <c r="G112" s="15" t="inlineStr">
         <is>
           <t>No te limites a decir que no hay y quedarte ahí, siempre hay un siguiente paso que ofrecer.</t>
         </is>
       </c>
-      <c r="H112" s="14" t="inlineStr">
+      <c r="H112" s="15" t="inlineStr">
         <is>
           <t>Si es una medicación que no puede interrumpirse, prioriza buscar en farmacias cercanas antes que pedir y esperar al día siguiente.</t>
         </is>
@@ -5141,312 +5449,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="74" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Por situación</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuántos mensajes hay de cada tipo y por dónde empezar con el equipo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Situación</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Mensajes</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Primera fila en 'Mensajes'</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Por dónde empezar</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Dudas sobre el genérico</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Fila 5</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Es la consulta que más veces se contesta distinto en la misma farmacia. Acordadla primero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Primera dispensación de un crónico</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Fila 14</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Aquí se juega la adherencia de los próximos meses. Vale la pena la versión larga.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>La novedad que ha visto en televisión o redes</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Fila 23</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>El riesgo es quedar por encima del paciente. Acordad el tono antes que el contenido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Cuando la respuesta es que no</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Fila 32</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>El momento que más desiguala a un equipo. Si solo escribís un bloque, que sea este.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Dejar de fumar</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Fila 41</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Consulta larga en un mostrador con cola: acordad cuándo se cita para otro momento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Complementos y probióticos</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Fila 50</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Cuidado con prometer. Revisad juntos la línea entre acompañar y colocar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Dermofarmacia y consulta de piel</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Fila 59</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Definid entre todos dónde está el límite para derivar al médico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>El precio y la comparación con internet</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Fila 68</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Se responde sin defenderse. Practicadlo en voz alta, cambia mucho.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>No lo tenemos ahora mismo</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Fila 77</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Lo importante no es la falta, es que el paciente se vaya sabiendo qué pasa y cuándo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Mayores y polimedicación</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Fila 86</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Bajad el ritmo y comprobad que se ha entendido. Es la parte que más se olvida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Cuando hay que derivar al médico</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Fila 95</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Acordad las señales de alarma por escrito. Es lo único que no admite estilo propio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Quejas y momentos incómodos</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Fila 104</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Reconocer el hecho no es dar la razón. Ensayadlo con dos personas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Total: 108 mensajes</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>